<commit_message>
Checkpoint Edge login and cover replacements
</commit_message>
<xml_diff>
--- a/Database/Market_Signal_Action_Queue.xlsx
+++ b/Database/Market_Signal_Action_Queue.xlsx
@@ -1943,7 +1943,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -14504,7 +14504,11 @@
       <c r="I272" t="b">
         <v>1</v>
       </c>
-      <c r="J272" t="inlineStr"/>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>406909884756</t>
+        </is>
+      </c>
       <c r="K272" t="inlineStr"/>
       <c r="L272" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Grey logic asset export packet
</commit_message>
<xml_diff>
--- a/Database/Market_Signal_Action_Queue.xlsx
+++ b/Database/Market_Signal_Action_Queue.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Queue'!$A$1:$L$275</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Queue'!$A$1:$L$283</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L275"/>
+  <dimension ref="A1:L283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2781,7 +2781,11 @@
           <t>406903249987</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>False</t>
@@ -2809,7 +2813,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2835,7 +2839,11 @@
           <t>406903250891</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>False</t>
@@ -2863,7 +2871,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2889,7 +2897,11 @@
           <t>406903252007</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>False</t>
@@ -4684,7 +4696,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0082</t>
+          <t>Acrylic-Grimdark-0001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4722,7 +4734,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>406902633400</t>
+          <t>406903249745</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -4742,7 +4754,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0083</t>
+          <t>Acrylic-Grimdark-0004</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4780,7 +4792,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>406902885214</t>
+          <t>406903250705</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -4800,7 +4812,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0085</t>
+          <t>Acrylic-Grimdark-0005</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4838,7 +4850,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>406903043482</t>
+          <t>406903251829</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -4858,7 +4870,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0002</t>
+          <t>Acrylic-Grimdark-0082</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4868,7 +4880,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4896,7 +4908,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>406902657898</t>
+          <t>406902633400</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -4906,7 +4918,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4928,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0003</t>
+          <t>Acrylic-Grimdark-0083</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4926,7 +4938,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4954,7 +4966,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>406902673249</t>
+          <t>406902885214</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -4974,7 +4986,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0005</t>
+          <t>Acrylic-Grimdark-0085</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4984,7 +4996,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -5012,7 +5024,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>406902893289</t>
+          <t>406903043482</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5032,7 +5044,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0007</t>
+          <t>Acrylic-Zen-0002</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -5070,7 +5082,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>406903028253</t>
+          <t>406902657898</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -5090,7 +5102,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0008</t>
+          <t>Acrylic-Zen-0003</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -5128,7 +5140,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>406903036452</t>
+          <t>406902673249</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -5148,7 +5160,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0009</t>
+          <t>Acrylic-Zen-0005</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -5186,7 +5198,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>406903047385</t>
+          <t>406902893289</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -5206,7 +5218,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0010</t>
+          <t>Acrylic-Zen-0007</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -5244,7 +5256,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>406903213858</t>
+          <t>406903028253</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -5254,7 +5266,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -5264,17 +5276,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Poster-Academia-0002</t>
+          <t>Acrylic-Zen-0008</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -5302,7 +5314,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>406902600741</t>
+          <t>406903036452</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -5322,17 +5334,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Poster-Academia-0005</t>
+          <t>Acrylic-Zen-0009</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -5360,7 +5372,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>406903038850</t>
+          <t>406903047385</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -5380,17 +5392,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Poster-Academia-0006</t>
+          <t>Acrylic-Zen-0010</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -5418,7 +5430,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>406903042690</t>
+          <t>406903213858</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -5428,7 +5440,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5450,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Poster-Academia-0008</t>
+          <t>Poster-Academia-0002</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5476,7 +5488,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>406903046097</t>
+          <t>406902600741</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -5486,7 +5498,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -5496,7 +5508,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Poster-Academia-0009</t>
+          <t>Poster-Academia-0005</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5534,7 +5546,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>406903209258</t>
+          <t>406903038850</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -5554,7 +5566,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Poster-Academia-0083</t>
+          <t>Poster-Academia-0006</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5592,7 +5604,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>406902669660</t>
+          <t>406903042690</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -5612,7 +5624,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Poster-Academia-0084</t>
+          <t>Poster-Academia-0008</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5650,7 +5662,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>406902691983</t>
+          <t>406903046097</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -5660,7 +5672,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -5670,7 +5682,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Poster-Academia-0091</t>
+          <t>Poster-Academia-0009</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5708,7 +5720,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>406902887127</t>
+          <t>406903209258</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -5718,7 +5730,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5740,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Poster-Zen-0001</t>
+          <t>Poster-Academia-0010</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5738,7 +5750,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5766,7 +5778,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>406902890971</t>
+          <t>406903249496</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -5786,7 +5798,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Poster-Zen-0002</t>
+          <t>Poster-Academia-0011</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5796,7 +5808,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5824,7 +5836,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>406902897663</t>
+          <t>406903250376</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -5844,7 +5856,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Poster-Zen-0004</t>
+          <t>Poster-Academia-0083</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5854,7 +5866,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5882,7 +5894,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>406903026999</t>
+          <t>406902669660</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -5902,7 +5914,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Poster-Zen-0005</t>
+          <t>Poster-Academia-0084</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5912,7 +5924,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5940,7 +5952,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>406903033377</t>
+          <t>406902691983</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -5960,12 +5972,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0004</t>
+          <t>Poster-Academia-0091</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5998,7 +6010,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>406892408950</t>
+          <t>406902887127</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -6008,7 +6020,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -6018,12 +6030,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0010</t>
+          <t>Poster-Zen-0001</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6056,7 +6068,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>406892414116</t>
+          <t>406902890971</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -6072,148 +6084,172 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0038</t>
+          <t>Poster-Zen-0002</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I106" t="b">
-        <v>0</v>
-      </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>406902897663</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0039</t>
+          <t>Poster-Zen-0004</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I107" t="b">
-        <v>0</v>
-      </c>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>406903026999</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0040</t>
+          <t>Poster-Zen-0005</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I108" t="b">
-        <v>0</v>
-      </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>406903033377</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L108" t="inlineStr">
         <is>
           <t>False</t>
@@ -6222,11 +6258,11 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0072</t>
+          <t>Sticker-Academia-0004</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6236,34 +6272,42 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I109" t="b">
-        <v>0</v>
-      </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>406892408950</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L109" t="inlineStr">
         <is>
           <t>False</t>
@@ -6272,11 +6316,11 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0073</t>
+          <t>Sticker-Zen-0010</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6291,29 +6335,37 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I110" t="b">
-        <v>0</v>
-      </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>406892414116</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L110" t="inlineStr">
         <is>
           <t>False</t>
@@ -6326,17 +6378,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0074</t>
+          <t>Acrylic-Grimdark-0038</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -6376,17 +6428,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0075</t>
+          <t>Acrylic-Grimdark-0039</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -6426,17 +6478,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0076</t>
+          <t>Acrylic-Grimdark-0040</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -6476,7 +6528,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0081</t>
+          <t>Sticker-Zen-0072</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6526,7 +6578,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0083</t>
+          <t>Sticker-Zen-0073</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6576,7 +6628,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0084</t>
+          <t>Sticker-Zen-0074</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6626,7 +6678,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0086</t>
+          <t>Sticker-Zen-0075</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -6676,7 +6728,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0087</t>
+          <t>Sticker-Zen-0076</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6726,7 +6778,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0088</t>
+          <t>Sticker-Zen-0081</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -6776,7 +6828,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0089</t>
+          <t>Sticker-Zen-0083</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -6826,7 +6878,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0091</t>
+          <t>Sticker-Zen-0084</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -6876,7 +6928,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0092</t>
+          <t>Sticker-Zen-0086</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -6926,7 +6978,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0093</t>
+          <t>Sticker-Zen-0087</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -6976,7 +7028,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0094</t>
+          <t>Sticker-Zen-0088</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7022,11 +7074,11 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0095</t>
+          <t>Sticker-Zen-0089</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7041,22 +7093,22 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Stable_Draft_Publish_When_Scheduled</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I125" t="b">
@@ -7072,11 +7124,11 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0096</t>
+          <t>Sticker-Zen-0091</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -7091,22 +7143,22 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Stable_Draft_Publish_When_Scheduled</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I126" t="b">
@@ -7122,11 +7174,11 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0097</t>
+          <t>Sticker-Zen-0092</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -7141,22 +7193,22 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Stable_Draft_Publish_When_Scheduled</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I127" t="b">
@@ -7172,11 +7224,11 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0098</t>
+          <t>Sticker-Zen-0093</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -7191,22 +7243,22 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Stable_Draft_Publish_When_Scheduled</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I128" t="b">
@@ -7222,11 +7274,11 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0099</t>
+          <t>Sticker-Zen-0094</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7241,22 +7293,22 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Stable_Draft_Publish_When_Scheduled</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I129" t="b">
@@ -7276,7 +7328,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0100</t>
+          <t>Sticker-Zen-0095</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -7326,7 +7378,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0101</t>
+          <t>Sticker-Zen-0096</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -7376,7 +7428,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0102</t>
+          <t>Sticker-Zen-0097</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7426,7 +7478,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0103</t>
+          <t>Sticker-Zen-0098</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -7476,7 +7528,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0104</t>
+          <t>Sticker-Zen-0099</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -7526,7 +7578,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0105</t>
+          <t>Sticker-Zen-0100</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7576,7 +7628,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0106</t>
+          <t>Sticker-Zen-0101</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7626,7 +7678,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0107</t>
+          <t>Sticker-Zen-0102</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7676,7 +7728,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0108</t>
+          <t>Sticker-Zen-0103</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7726,7 +7778,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0109</t>
+          <t>Sticker-Zen-0104</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7776,7 +7828,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0110</t>
+          <t>Sticker-Zen-0105</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7826,7 +7878,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0111</t>
+          <t>Sticker-Zen-0106</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7876,7 +7928,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0112</t>
+          <t>Sticker-Zen-0107</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7926,7 +7978,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0113</t>
+          <t>Sticker-Zen-0108</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -7976,7 +8028,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0114</t>
+          <t>Sticker-Zen-0109</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8026,7 +8078,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0115</t>
+          <t>Sticker-Zen-0110</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8076,7 +8128,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0117</t>
+          <t>Sticker-Zen-0111</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8126,7 +8178,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0123</t>
+          <t>Sticker-Zen-0112</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8176,7 +8228,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0126</t>
+          <t>Sticker-Zen-0113</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -8226,7 +8278,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0127</t>
+          <t>Sticker-Zen-0114</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -8276,7 +8328,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0128</t>
+          <t>Sticker-Zen-0115</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -8326,7 +8378,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0129</t>
+          <t>Sticker-Zen-0117</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -8376,7 +8428,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0130</t>
+          <t>Sticker-Zen-0123</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -8426,7 +8478,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0131</t>
+          <t>Sticker-Zen-0126</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -8476,7 +8528,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0132</t>
+          <t>Sticker-Zen-0127</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -8526,7 +8578,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0133</t>
+          <t>Sticker-Zen-0128</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -8576,7 +8628,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0134</t>
+          <t>Sticker-Zen-0129</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -8626,7 +8678,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0135</t>
+          <t>Sticker-Zen-0130</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -8676,7 +8728,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0136</t>
+          <t>Sticker-Zen-0131</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -8726,7 +8778,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0138</t>
+          <t>Sticker-Zen-0132</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8776,7 +8828,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0139</t>
+          <t>Sticker-Zen-0133</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8826,7 +8878,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0150</t>
+          <t>Sticker-Zen-0134</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -8876,7 +8928,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0151</t>
+          <t>Sticker-Zen-0135</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8926,7 +8978,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0153</t>
+          <t>Sticker-Zen-0136</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -8976,7 +9028,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0154</t>
+          <t>Sticker-Zen-0138</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -9026,7 +9078,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0155</t>
+          <t>Sticker-Zen-0139</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -9076,7 +9128,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0156</t>
+          <t>Sticker-Zen-0150</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -9126,7 +9178,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0157</t>
+          <t>Sticker-Zen-0151</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -9176,7 +9228,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0158</t>
+          <t>Sticker-Zen-0153</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -9226,7 +9278,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0159</t>
+          <t>Sticker-Zen-0154</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -9276,7 +9328,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0160</t>
+          <t>Sticker-Zen-0155</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -9322,95 +9374,91 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Poster-Academia-0011</t>
+          <t>Sticker-Zen-0156</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I171" t="b">
         <v>0</v>
       </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t>406903250376</t>
-        </is>
-      </c>
+      <c r="J171" t="inlineStr"/>
       <c r="K171" t="inlineStr"/>
       <c r="L171" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Poster-Academia-0013</t>
+          <t>Sticker-Zen-0157</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I172" t="b">
@@ -9420,47 +9468,47 @@
       <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Poster-Academia-0026</t>
+          <t>Sticker-Zen-0158</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I173" t="b">
@@ -9470,47 +9518,47 @@
       <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Poster-Academia-0027</t>
+          <t>Sticker-Zen-0159</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I174" t="b">
@@ -9520,47 +9568,47 @@
       <c r="K174" t="inlineStr"/>
       <c r="L174" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Poster-Academia-0028</t>
+          <t>Sticker-Zen-0160</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I175" t="b">
@@ -9570,22 +9618,22 @@
       <c r="K175" t="inlineStr"/>
       <c r="L175" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Acrylic-Academia-0001</t>
+          <t>Poster-Academia-0013</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -9595,37 +9643,29 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Item has at least one view; do not churn copy too quickly.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I176" t="b">
-        <v>1</v>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t>406902588642</t>
-        </is>
-      </c>
-      <c r="K176" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
       <c r="L176" t="inlineStr">
         <is>
           <t>True</t>
@@ -9634,114 +9674,98 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0004</t>
+          <t>Poster-Academia-0026</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Item has at least one view; do not churn copy too quickly.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I177" t="b">
-        <v>1</v>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t>406902888077</t>
-        </is>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
       <c r="L177" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0006</t>
+          <t>Poster-Academia-0027</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Item has at least one view; do not churn copy too quickly.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I178" t="b">
-        <v>1</v>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>406902898909</t>
-        </is>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr">
         <is>
           <t>True</t>
@@ -9750,11 +9774,11 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Poster-Academia-0081</t>
+          <t>Poster-Academia-0028</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -9769,37 +9793,29 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Published_Has_View_Monitor</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Item has at least one view; do not churn copy too quickly.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I179" t="b">
-        <v>1</v>
-      </c>
-      <c r="J179" t="inlineStr">
-        <is>
-          <t>406902627420</t>
-        </is>
-      </c>
-      <c r="K179" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
       <c r="L179" t="inlineStr">
         <is>
           <t>True</t>
@@ -9812,12 +9828,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Poster-Academia-0082</t>
+          <t>Acrylic-Academia-0001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -9850,17 +9866,17 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>406902648209</t>
+          <t>406902588642</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -9870,17 +9886,17 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Poster-Academia-0085</t>
+          <t>Acrylic-Zen-0004</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -9908,7 +9924,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>406902882943</t>
+          <t>406902888077</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -9924,11 +9940,11 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0001</t>
+          <t>Acrylic-Zen-0006</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -9938,27 +9954,27 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>No safe action under current weak-network protocol.</t>
+          <t>Item has at least one view; do not churn copy too quickly.</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I182" t="b">
@@ -9966,53 +9982,57 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>406903249745</t>
-        </is>
-      </c>
-      <c r="K182" t="inlineStr"/>
+          <t>406902898909</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0004</t>
+          <t>Poster-Academia-0081</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>No safe action under current weak-network protocol.</t>
+          <t>Item has at least one view; do not churn copy too quickly.</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I183" t="b">
@@ -10020,53 +10040,57 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>406903250705</t>
-        </is>
-      </c>
-      <c r="K183" t="inlineStr"/>
+          <t>406902627420</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0005</t>
+          <t>Poster-Academia-0082</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>No safe action under current weak-network protocol.</t>
+          <t>Item has at least one view; do not churn copy too quickly.</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I184" t="b">
@@ -10074,10 +10098,14 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>406903251829</t>
-        </is>
-      </c>
-      <c r="K184" t="inlineStr"/>
+          <t>406902648209</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="L184" t="inlineStr">
         <is>
           <t>False</t>
@@ -10086,41 +10114,41 @@
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0006</t>
+          <t>Poster-Academia-0085</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Has_View_Monitor</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>MONITOR_FOR_CLICK_OR_FAVORITE_SIGNAL</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>No safe action under current weak-network protocol.</t>
+          <t>Item has at least one view; do not churn copy too quickly.</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I185" t="b">
@@ -10128,10 +10156,14 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>406903252506</t>
-        </is>
-      </c>
-      <c r="K185" t="inlineStr"/>
+          <t>406902882943</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L185" t="inlineStr">
         <is>
           <t>False</t>
@@ -10144,7 +10176,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0007</t>
+          <t>Acrylic-Grimdark-0006</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -10182,7 +10214,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>406903731967</t>
+          <t>406903252506</t>
         </is>
       </c>
       <c r="K186" t="inlineStr"/>
@@ -10198,7 +10230,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0008</t>
+          <t>Acrylic-Grimdark-0007</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -10236,7 +10268,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>406903746215</t>
+          <t>406903731967</t>
         </is>
       </c>
       <c r="K187" t="inlineStr"/>
@@ -10252,7 +10284,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0009</t>
+          <t>Acrylic-Grimdark-0008</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -10290,7 +10322,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>406903749989</t>
+          <t>406903746215</t>
         </is>
       </c>
       <c r="K188" t="inlineStr"/>
@@ -10306,7 +10338,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0010</t>
+          <t>Acrylic-Grimdark-0009</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -10344,7 +10376,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>406903756190</t>
+          <t>406903749989</t>
         </is>
       </c>
       <c r="K189" t="inlineStr"/>
@@ -10360,7 +10392,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0011</t>
+          <t>Acrylic-Grimdark-0010</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -10396,7 +10428,11 @@
       <c r="I190" t="b">
         <v>1</v>
       </c>
-      <c r="J190" t="inlineStr"/>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>406903756190</t>
+        </is>
+      </c>
       <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr">
         <is>
@@ -10410,7 +10446,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0012</t>
+          <t>Acrylic-Grimdark-0011</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -10460,7 +10496,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0013</t>
+          <t>Acrylic-Grimdark-0012</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -10510,7 +10546,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0014</t>
+          <t>Acrylic-Grimdark-0013</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -10560,7 +10596,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0015</t>
+          <t>Acrylic-Grimdark-0014</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -10610,7 +10646,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0016</t>
+          <t>Acrylic-Grimdark-0015</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -10660,7 +10696,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0017</t>
+          <t>Acrylic-Grimdark-0016</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -10710,7 +10746,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0018</t>
+          <t>Acrylic-Grimdark-0017</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -10760,7 +10796,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0019</t>
+          <t>Acrylic-Grimdark-0018</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -10810,7 +10846,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0021</t>
+          <t>Acrylic-Grimdark-0019</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -10860,7 +10896,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0022</t>
+          <t>Acrylic-Grimdark-0021</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -10910,7 +10946,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0023</t>
+          <t>Acrylic-Grimdark-0022</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -10960,7 +10996,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0024</t>
+          <t>Acrylic-Grimdark-0023</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -11010,7 +11046,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0025</t>
+          <t>Acrylic-Grimdark-0024</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -11060,7 +11096,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0026</t>
+          <t>Acrylic-Grimdark-0025</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -11110,7 +11146,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0027</t>
+          <t>Acrylic-Grimdark-0026</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -11160,7 +11196,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0028</t>
+          <t>Acrylic-Grimdark-0027</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -11210,7 +11246,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0030</t>
+          <t>Acrylic-Grimdark-0028</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -11260,7 +11296,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0031</t>
+          <t>Acrylic-Grimdark-0030</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -11310,7 +11346,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0032</t>
+          <t>Acrylic-Grimdark-0031</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -11360,7 +11396,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0033</t>
+          <t>Acrylic-Grimdark-0032</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -11410,7 +11446,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0034</t>
+          <t>Acrylic-Grimdark-0033</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -11460,7 +11496,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0035</t>
+          <t>Acrylic-Grimdark-0034</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -11510,7 +11546,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0036</t>
+          <t>Acrylic-Grimdark-0035</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -11560,7 +11596,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0037</t>
+          <t>Acrylic-Grimdark-0036</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -11610,17 +11646,17 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Poster-Academia-0010</t>
+          <t>Acrylic-Grimdark-0037</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -11646,11 +11682,7 @@
       <c r="I215" t="b">
         <v>1</v>
       </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t>406903249496</t>
-        </is>
-      </c>
+      <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr"/>
       <c r="L215" t="inlineStr">
         <is>
@@ -14522,7 +14554,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0048</t>
+          <t>Sticker-Zen-0045-FIX1</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -14558,7 +14590,11 @@
       <c r="I273" t="b">
         <v>1</v>
       </c>
-      <c r="J273" t="inlineStr"/>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>406909890800</t>
+        </is>
+      </c>
       <c r="K273" t="inlineStr"/>
       <c r="L273" t="inlineStr">
         <is>
@@ -14572,7 +14608,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0067</t>
+          <t>Sticker-Zen-0046-FIX1</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -14608,7 +14644,11 @@
       <c r="I274" t="b">
         <v>1</v>
       </c>
-      <c r="J274" t="inlineStr"/>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>406909891985</t>
+        </is>
+      </c>
       <c r="K274" t="inlineStr"/>
       <c r="L274" t="inlineStr">
         <is>
@@ -14622,7 +14662,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0068</t>
+          <t>Sticker-Zen-0048</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -14666,8 +14706,432 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>20</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0049-FIX1</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I276" t="b">
+        <v>1</v>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>406909893702</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr"/>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>20</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0050-FIX1</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I277" t="b">
+        <v>1</v>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>406909904704</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr"/>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>20</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0051-FIX1</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I278" t="b">
+        <v>1</v>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>406909905683</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr"/>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>20</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0052-FIX1</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I279" t="b">
+        <v>1</v>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>406909906686</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr"/>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>20</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0053-FIX1</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I280" t="b">
+        <v>1</v>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>406909907111</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr"/>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>20</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0054-FIX1</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I281" t="b">
+        <v>1</v>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>406909907742</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr"/>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>20</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0067</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I282" t="b">
+        <v>1</v>
+      </c>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="inlineStr"/>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>20</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0068</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>No safe action under current weak-network protocol.</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="I283" t="b">
+        <v>1</v>
+      </c>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="inlineStr"/>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L275"/>
+  <autoFilter ref="A1:L283"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Printify self healing daemon
</commit_message>
<xml_diff>
--- a/Database/Market_Signal_Action_Queue.xlsx
+++ b/Database/Market_Signal_Action_Queue.xlsx
@@ -5856,7 +5856,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Poster-Academia-0083</t>
+          <t>Poster-Academia-0013</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>406902669660</t>
+          <t>406903251282</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Poster-Academia-0084</t>
+          <t>Poster-Academia-0083</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>406902691983</t>
+          <t>406902669660</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Poster-Academia-0091</t>
+          <t>Poster-Academia-0084</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>406902887127</t>
+          <t>406902691983</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Poster-Zen-0001</t>
+          <t>Poster-Academia-0091</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6040,7 +6040,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -6068,7 +6068,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>406902890971</t>
+          <t>406902887127</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -6088,7 +6088,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Poster-Zen-0002</t>
+          <t>Poster-Zen-0001</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>406902897663</t>
+          <t>406902890971</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -6136,7 +6136,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Poster-Zen-0004</t>
+          <t>Poster-Zen-0002</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6184,7 +6184,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>406903026999</t>
+          <t>406902897663</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Poster-Zen-0005</t>
+          <t>Poster-Zen-0004</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>406903033377</t>
+          <t>406903026999</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -6252,7 +6252,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -6262,17 +6262,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0004</t>
+          <t>Poster-Zen-0005</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -6300,7 +6300,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>406892408950</t>
+          <t>406903033377</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0010</t>
+          <t>Sticker-Academia-0004</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>406892414116</t>
+          <t>406892408950</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -6374,48 +6374,56 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0038</t>
+          <t>Sticker-Zen-0010</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I111" t="b">
-        <v>0</v>
-      </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>406892414116</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L111" t="inlineStr">
         <is>
           <t>False</t>
@@ -6428,7 +6436,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0039</t>
+          <t>Acrylic-Grimdark-0038</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6478,7 +6486,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0040</t>
+          <t>Acrylic-Grimdark-0039</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6528,17 +6536,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0072</t>
+          <t>Acrylic-Grimdark-0040</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -6578,7 +6586,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0073</t>
+          <t>Sticker-Zen-0072</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6628,7 +6636,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0074</t>
+          <t>Sticker-Zen-0073</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6678,7 +6686,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0075</t>
+          <t>Sticker-Zen-0074</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -6728,7 +6736,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0076</t>
+          <t>Sticker-Zen-0075</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6778,7 +6786,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0081</t>
+          <t>Sticker-Zen-0076</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -6828,7 +6836,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0083</t>
+          <t>Sticker-Zen-0081</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -6878,7 +6886,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0084</t>
+          <t>Sticker-Zen-0083</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -6928,7 +6936,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0086</t>
+          <t>Sticker-Zen-0084</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -6978,7 +6986,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0087</t>
+          <t>Sticker-Zen-0086</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -7028,7 +7036,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0088</t>
+          <t>Sticker-Zen-0087</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7078,7 +7086,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0089</t>
+          <t>Sticker-Zen-0088</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7128,7 +7136,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0091</t>
+          <t>Sticker-Zen-0089</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -7178,7 +7186,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0092</t>
+          <t>Sticker-Zen-0091</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -7228,7 +7236,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0093</t>
+          <t>Sticker-Zen-0092</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -7278,7 +7286,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0094</t>
+          <t>Sticker-Zen-0093</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7324,11 +7332,11 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0095</t>
+          <t>Sticker-Zen-0094</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -7343,22 +7351,22 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Stable_Draft_Publish_When_Scheduled</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I130" t="b">
@@ -7378,7 +7386,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0096</t>
+          <t>Sticker-Zen-0095</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -7428,7 +7436,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0097</t>
+          <t>Sticker-Zen-0096</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7478,7 +7486,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0098</t>
+          <t>Sticker-Zen-0097</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -7528,7 +7536,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0099</t>
+          <t>Sticker-Zen-0098</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -7578,7 +7586,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0100</t>
+          <t>Sticker-Zen-0099</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7628,7 +7636,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0101</t>
+          <t>Sticker-Zen-0100</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7678,7 +7686,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0102</t>
+          <t>Sticker-Zen-0101</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7728,7 +7736,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0103</t>
+          <t>Sticker-Zen-0102</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7778,7 +7786,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0104</t>
+          <t>Sticker-Zen-0103</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7828,7 +7836,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0105</t>
+          <t>Sticker-Zen-0104</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7878,7 +7886,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0106</t>
+          <t>Sticker-Zen-0105</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7928,7 +7936,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0107</t>
+          <t>Sticker-Zen-0106</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7978,7 +7986,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0108</t>
+          <t>Sticker-Zen-0107</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -8028,7 +8036,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0109</t>
+          <t>Sticker-Zen-0108</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8078,7 +8086,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0110</t>
+          <t>Sticker-Zen-0109</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8128,7 +8136,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0111</t>
+          <t>Sticker-Zen-0110</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8178,7 +8186,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0112</t>
+          <t>Sticker-Zen-0111</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8228,7 +8236,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0113</t>
+          <t>Sticker-Zen-0112</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -8278,7 +8286,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0114</t>
+          <t>Sticker-Zen-0113</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -8328,7 +8336,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0115</t>
+          <t>Sticker-Zen-0114</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -8378,7 +8386,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0117</t>
+          <t>Sticker-Zen-0115</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -8428,7 +8436,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0123</t>
+          <t>Sticker-Zen-0117</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -8478,7 +8486,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0126</t>
+          <t>Sticker-Zen-0123</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -8528,7 +8536,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0127</t>
+          <t>Sticker-Zen-0126</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -8578,7 +8586,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0128</t>
+          <t>Sticker-Zen-0127</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -8628,7 +8636,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0129</t>
+          <t>Sticker-Zen-0128</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -8678,7 +8686,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0130</t>
+          <t>Sticker-Zen-0129</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -8728,7 +8736,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0131</t>
+          <t>Sticker-Zen-0130</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -8778,7 +8786,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0132</t>
+          <t>Sticker-Zen-0131</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8828,7 +8836,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0133</t>
+          <t>Sticker-Zen-0132</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8878,7 +8886,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0134</t>
+          <t>Sticker-Zen-0133</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -8928,7 +8936,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0135</t>
+          <t>Sticker-Zen-0134</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8978,7 +8986,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0136</t>
+          <t>Sticker-Zen-0135</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -9028,7 +9036,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0138</t>
+          <t>Sticker-Zen-0136</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -9078,7 +9086,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0139</t>
+          <t>Sticker-Zen-0138</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -9128,7 +9136,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0150</t>
+          <t>Sticker-Zen-0139</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -9178,7 +9186,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0151</t>
+          <t>Sticker-Zen-0150</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -9228,7 +9236,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0153</t>
+          <t>Sticker-Zen-0151</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -9278,7 +9286,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0154</t>
+          <t>Sticker-Zen-0153</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -9328,7 +9336,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0155</t>
+          <t>Sticker-Zen-0154</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -9378,7 +9386,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0156</t>
+          <t>Sticker-Zen-0155</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -9428,7 +9436,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0157</t>
+          <t>Sticker-Zen-0156</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -9478,7 +9486,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0158</t>
+          <t>Sticker-Zen-0157</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -9528,7 +9536,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0159</t>
+          <t>Sticker-Zen-0158</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -9578,7 +9586,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0160</t>
+          <t>Sticker-Zen-0159</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -9624,41 +9632,41 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Poster-Academia-0013</t>
+          <t>Sticker-Zen-0160</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I176" t="b">
@@ -9668,7 +9676,7 @@
       <c r="K176" t="inlineStr"/>
       <c r="L176" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -10482,7 +10490,11 @@
       <c r="I191" t="b">
         <v>1</v>
       </c>
-      <c r="J191" t="inlineStr"/>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>406903760725</t>
+        </is>
+      </c>
       <c r="K191" t="inlineStr"/>
       <c r="L191" t="inlineStr">
         <is>
@@ -10532,7 +10544,11 @@
       <c r="I192" t="b">
         <v>1</v>
       </c>
-      <c r="J192" t="inlineStr"/>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>406909148324</t>
+        </is>
+      </c>
       <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr">
         <is>
@@ -10582,7 +10598,11 @@
       <c r="I193" t="b">
         <v>1</v>
       </c>
-      <c r="J193" t="inlineStr"/>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>406909151733</t>
+        </is>
+      </c>
       <c r="K193" t="inlineStr"/>
       <c r="L193" t="inlineStr">
         <is>
@@ -10632,7 +10652,11 @@
       <c r="I194" t="b">
         <v>1</v>
       </c>
-      <c r="J194" t="inlineStr"/>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>406909159060</t>
+        </is>
+      </c>
       <c r="K194" t="inlineStr"/>
       <c r="L194" t="inlineStr">
         <is>
@@ -10682,7 +10706,11 @@
       <c r="I195" t="b">
         <v>1</v>
       </c>
-      <c r="J195" t="inlineStr"/>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>406909166683</t>
+        </is>
+      </c>
       <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr">
         <is>
@@ -11732,7 +11760,11 @@
       <c r="I216" t="b">
         <v>1</v>
       </c>
-      <c r="J216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>406903252244</t>
+        </is>
+      </c>
       <c r="K216" t="inlineStr"/>
       <c r="L216" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add quiet jade pivot and grunt engine
</commit_message>
<xml_diff>
--- a/Database/Market_Signal_Action_Queue.xlsx
+++ b/Database/Market_Signal_Action_Queue.xlsx
@@ -3130,12 +3130,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Poster-Academia-0021</t>
+          <t>Acrylic-Academia-0003</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Local QA issue: corrupt_production</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3166,11 +3166,19 @@
       <c r="I51" t="b">
         <v>1</v>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>406902703464</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -3180,12 +3188,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0001</t>
+          <t>Acrylic-Academia-0005</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3195,7 +3203,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3205,7 +3213,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3216,11 +3224,19 @@
       <c r="I52" t="b">
         <v>1</v>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>406903039716</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -3230,22 +3246,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0002</t>
+          <t>Acrylic-Grimdark-0001</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3255,7 +3271,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3266,8 +3282,16 @@
       <c r="I53" t="b">
         <v>1</v>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>406903249745</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>False</t>
@@ -3280,22 +3304,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0003</t>
+          <t>Acrylic-Grimdark-0004</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3305,7 +3329,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3316,8 +3340,16 @@
       <c r="I54" t="b">
         <v>1</v>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>406903250705</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>False</t>
@@ -3330,22 +3362,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0005-FIX2</t>
+          <t>Acrylic-Grimdark-0005</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Fix_Gallery_First</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3355,7 +3387,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3366,8 +3398,16 @@
       <c r="I55" t="b">
         <v>1</v>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>406903251829</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>False</t>
@@ -3380,22 +3420,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0013</t>
+          <t>Acrylic-Grimdark-0082</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3405,7 +3445,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3416,8 +3456,16 @@
       <c r="I56" t="b">
         <v>1</v>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>406902633400</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>False</t>
@@ -3430,22 +3478,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0006</t>
+          <t>Acrylic-Grimdark-0083</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3455,7 +3503,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3466,8 +3514,16 @@
       <c r="I57" t="b">
         <v>1</v>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>406902885214</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>False</t>
@@ -3480,22 +3536,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0021</t>
+          <t>Acrylic-Grimdark-0085</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3505,7 +3561,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3516,8 +3572,16 @@
       <c r="I58" t="b">
         <v>1</v>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>406903043482</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>False</t>
@@ -3530,12 +3594,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0023</t>
+          <t>Acrylic-Zen-0002</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3545,7 +3609,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3555,7 +3619,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3566,11 +3630,19 @@
       <c r="I59" t="b">
         <v>1</v>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>406902657898</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -3580,12 +3652,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0028</t>
+          <t>Acrylic-Zen-0003</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3595,7 +3667,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3605,7 +3677,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3616,8 +3688,16 @@
       <c r="I60" t="b">
         <v>1</v>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>406902673249</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>False</t>
@@ -3630,12 +3710,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0030</t>
+          <t>Acrylic-Zen-0005</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3645,7 +3725,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3655,7 +3735,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3666,8 +3746,16 @@
       <c r="I61" t="b">
         <v>1</v>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>406902893289</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>False</t>
@@ -3680,12 +3768,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0033</t>
+          <t>Acrylic-Zen-0007</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3695,7 +3783,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3705,7 +3793,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3716,11 +3804,19 @@
       <c r="I62" t="b">
         <v>1</v>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>406903028253</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -3730,12 +3826,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0039</t>
+          <t>Acrylic-Zen-0008</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3745,7 +3841,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3755,7 +3851,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3766,8 +3862,16 @@
       <c r="I63" t="b">
         <v>1</v>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>406903036452</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>False</t>
@@ -3780,12 +3884,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0078</t>
+          <t>Acrylic-Zen-0009</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3795,7 +3899,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3805,7 +3909,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3816,8 +3920,16 @@
       <c r="I64" t="b">
         <v>1</v>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>406903047385</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>False</t>
@@ -3830,12 +3942,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0079</t>
+          <t>Acrylic-Zen-0010</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3845,7 +3957,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3855,7 +3967,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3866,8 +3978,16 @@
       <c r="I65" t="b">
         <v>1</v>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>406903213858</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L65" t="inlineStr">
         <is>
           <t>False</t>
@@ -3880,22 +4000,22 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0080</t>
+          <t>Poster-Academia-0002</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3905,7 +4025,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3916,8 +4036,16 @@
       <c r="I66" t="b">
         <v>1</v>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>406902600741</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>False</t>
@@ -3930,22 +4058,22 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0082</t>
+          <t>Poster-Academia-0005</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3955,7 +4083,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3966,8 +4094,16 @@
       <c r="I67" t="b">
         <v>1</v>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>406903038850</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L67" t="inlineStr">
         <is>
           <t>False</t>
@@ -3980,22 +4116,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0085</t>
+          <t>Poster-Academia-0006</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -4005,7 +4141,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -4016,11 +4152,19 @@
       <c r="I68" t="b">
         <v>1</v>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>406903042690</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4030,22 +4174,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0090</t>
+          <t>Poster-Academia-0008</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -4055,7 +4199,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -4066,11 +4210,19 @@
       <c r="I69" t="b">
         <v>1</v>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>406903046097</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4080,22 +4232,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0116</t>
+          <t>Poster-Academia-0009</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4105,7 +4257,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -4116,8 +4268,16 @@
       <c r="I70" t="b">
         <v>1</v>
       </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>406903209258</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
           <t>False</t>
@@ -4130,22 +4290,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0118</t>
+          <t>Poster-Academia-0010</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4155,7 +4315,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4166,8 +4326,16 @@
       <c r="I71" t="b">
         <v>1</v>
       </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>406903249496</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L71" t="inlineStr">
         <is>
           <t>False</t>
@@ -4180,22 +4348,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0120</t>
+          <t>Poster-Academia-0011</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -4205,7 +4373,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -4216,11 +4384,19 @@
       <c r="I72" t="b">
         <v>1</v>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>406903250376</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4230,22 +4406,22 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0121</t>
+          <t>Poster-Academia-0013</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4255,7 +4431,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -4266,11 +4442,19 @@
       <c r="I73" t="b">
         <v>1</v>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>406903251282</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4280,22 +4464,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0122</t>
+          <t>Poster-Academia-0021</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4305,7 +4489,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: corrupt_production</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -4320,7 +4504,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4330,22 +4514,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0124</t>
+          <t>Poster-Academia-0083</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4355,7 +4539,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4366,11 +4550,19 @@
       <c r="I75" t="b">
         <v>1</v>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>406902669660</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4380,22 +4572,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0125</t>
+          <t>Poster-Academia-0084</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4405,7 +4597,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4416,8 +4608,16 @@
       <c r="I76" t="b">
         <v>1</v>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>406902691983</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
           <t>False</t>
@@ -4430,22 +4630,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0140</t>
+          <t>Poster-Academia-0091</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4455,7 +4655,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -4466,11 +4666,19 @@
       <c r="I77" t="b">
         <v>1</v>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>406902887127</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -4480,12 +4688,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0144</t>
+          <t>Poster-Zen-0001</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4495,7 +4703,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4505,7 +4713,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -4516,8 +4724,16 @@
       <c r="I78" t="b">
         <v>1</v>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>406902890971</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr">
         <is>
           <t>False</t>
@@ -4530,12 +4746,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0152</t>
+          <t>Poster-Zen-0002</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4545,7 +4761,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Published_Zero_View_Copy_Ad_Review</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4555,7 +4771,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Local QA issue: missing_cover; missing_gallery</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4566,31 +4782,39 @@
       <c r="I79" t="b">
         <v>1</v>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>406902897663</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Acrylic-Academia-0003</t>
+          <t>Poster-Zen-0004</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4600,17 +4824,17 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I80" t="b">
@@ -4618,7 +4842,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>406902703464</t>
+          <t>406903026999</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -4628,27 +4852,27 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Acrylic-Academia-0005</t>
+          <t>Poster-Zen-0005</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4658,17 +4882,17 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_image_note</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I81" t="b">
@@ -4676,7 +4900,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>406903039716</t>
+          <t>406903033377</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -4686,62 +4910,54 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0001</t>
+          <t>Sticker-Academia-0001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>406903249745</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
           <t>False</t>
@@ -4750,56 +4966,48 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0004</t>
+          <t>Sticker-Academia-0002</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I83" t="b">
         <v>1</v>
       </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>406903250705</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
           <t>False</t>
@@ -4808,56 +5016,48 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0005</t>
+          <t>Sticker-Academia-0003</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I84" t="b">
         <v>1</v>
       </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>406903251829</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
           <t>False</t>
@@ -4866,56 +5066,48 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0082</t>
+          <t>Sticker-Academia-0005-FIX2</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Fix_Gallery_First</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_gallery</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I85" t="b">
         <v>1</v>
       </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>406902633400</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>False</t>
@@ -4924,56 +5116,48 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0083</t>
+          <t>Sticker-Academia-0013</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I86" t="b">
         <v>1</v>
       </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>406902885214</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>False</t>
@@ -4982,56 +5166,48 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0085</t>
+          <t>Sticker-Zen-0006</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I87" t="b">
         <v>1</v>
       </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>406903043482</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>False</t>
@@ -5040,16 +5216,16 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0002</t>
+          <t>Sticker-Zen-0021</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5059,55 +5235,47 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I88" t="b">
         <v>1</v>
       </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>406902657898</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0003</t>
+          <t>Sticker-Zen-0023</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5117,37 +5285,29 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I89" t="b">
         <v>1</v>
       </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>406902673249</t>
-        </is>
-      </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>False</t>
@@ -5156,16 +5316,16 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0005</t>
+          <t>Sticker-Zen-0028</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5175,37 +5335,29 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I90" t="b">
         <v>1</v>
       </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>406902893289</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>False</t>
@@ -5214,16 +5366,16 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0007</t>
+          <t>Sticker-Zen-0030</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5233,55 +5385,47 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I91" t="b">
         <v>1</v>
       </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>406903028253</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0008</t>
+          <t>Sticker-Zen-0033</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5291,37 +5435,29 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I92" t="b">
         <v>1</v>
       </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>406903036452</t>
-        </is>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>False</t>
@@ -5330,16 +5466,16 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0009</t>
+          <t>Sticker-Zen-0039</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -5349,37 +5485,29 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I93" t="b">
         <v>1</v>
       </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>406903047385</t>
-        </is>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
           <t>False</t>
@@ -5388,16 +5516,16 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0010</t>
+          <t>Sticker-Zen-0078</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5407,37 +5535,29 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I94" t="b">
         <v>1</v>
       </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>406903213858</t>
-        </is>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>False</t>
@@ -5446,56 +5566,48 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Poster-Academia-0002</t>
+          <t>Sticker-Zen-0079</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I95" t="b">
         <v>1</v>
       </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>406902600741</t>
-        </is>
-      </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>False</t>
@@ -5504,56 +5616,48 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Poster-Academia-0005</t>
+          <t>Sticker-Zen-0080</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I96" t="b">
         <v>1</v>
       </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>406903038850</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>False</t>
@@ -5562,172 +5666,148 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Poster-Academia-0006</t>
+          <t>Sticker-Zen-0082</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I97" t="b">
         <v>1</v>
       </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>406903042690</t>
-        </is>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Poster-Academia-0008</t>
+          <t>Sticker-Zen-0085</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I98" t="b">
         <v>1</v>
       </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>406903046097</t>
-        </is>
-      </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Poster-Academia-0009</t>
+          <t>Sticker-Zen-0090</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I99" t="b">
         <v>1</v>
       </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>406903209258</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>False</t>
@@ -5736,56 +5816,48 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Poster-Academia-0010</t>
+          <t>Sticker-Zen-0116</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I100" t="b">
         <v>1</v>
       </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>406903249496</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>False</t>
@@ -5794,230 +5866,198 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Poster-Academia-0011</t>
+          <t>Sticker-Zen-0118</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I101" t="b">
         <v>1</v>
       </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>406903250376</t>
-        </is>
-      </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Poster-Academia-0013</t>
+          <t>Sticker-Zen-0120</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I102" t="b">
         <v>1</v>
       </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>406903251282</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Poster-Academia-0083</t>
+          <t>Sticker-Zen-0121</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I103" t="b">
         <v>1</v>
       </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t>406902669660</t>
-        </is>
-      </c>
-      <c r="K103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Poster-Academia-0084</t>
+          <t>Sticker-Zen-0122</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I104" t="b">
         <v>1</v>
       </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>406902691983</t>
-        </is>
-      </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>False</t>
@@ -6026,74 +6066,66 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Poster-Academia-0091</t>
+          <t>Sticker-Zen-0124</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I105" t="b">
         <v>1</v>
       </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>406902887127</t>
-        </is>
-      </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Poster-Zen-0001</t>
+          <t>Sticker-Zen-0125</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6103,37 +6135,29 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I106" t="b">
         <v>1</v>
       </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>406902890971</t>
-        </is>
-      </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>False</t>
@@ -6142,16 +6166,16 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Poster-Zen-0002</t>
+          <t>Sticker-Zen-0140</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6161,55 +6185,47 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I107" t="b">
         <v>1</v>
       </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>406902897663</t>
-        </is>
-      </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Poster-Zen-0004</t>
+          <t>Sticker-Zen-0144</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6219,55 +6235,47 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I108" t="b">
         <v>1</v>
       </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>406903026999</t>
-        </is>
-      </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Poster-Zen-0005</t>
+          <t>Sticker-Zen-0152</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6277,37 +6285,29 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Published_Zero_View_Copy_Ad_Review</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>WAIT_24H_AFTER_2PCT_ADS_THEN_APPLY_COPY_TEST</t>
+          <t>QA_HOLD_OR_REBUILD</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Published item has 0 visible views in last Seller Hub snapshot; 2% General ads are active, so wait for a cleaner baseline before editing online.</t>
+          <t>Local QA issue: missing_cover; missing_gallery</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I109" t="b">
         <v>1</v>
       </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>406903033377</t>
-        </is>
-      </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>False</t>

</xml_diff>

<commit_message>
Refresh local factory maintenance state
</commit_message>
<xml_diff>
--- a/Database/Market_Signal_Action_Queue.xlsx
+++ b/Database/Market_Signal_Action_Queue.xlsx
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0072</t>
+          <t>Sticker-Zen-0075</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0073</t>
+          <t>Sticker-Zen-0076</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0074</t>
+          <t>Sticker-Zen-0081</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0075</t>
+          <t>Sticker-Zen-0083</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0076</t>
+          <t>Sticker-Zen-0084</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0081</t>
+          <t>Sticker-Zen-0086</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0083</t>
+          <t>Sticker-Zen-0087</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0084</t>
+          <t>Sticker-Zen-0088</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0086</t>
+          <t>Sticker-Zen-0089</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0087</t>
+          <t>Sticker-Zen-0091</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0088</t>
+          <t>Sticker-Zen-0092</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6040,7 +6040,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0089</t>
+          <t>Sticker-Zen-0093</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0091</t>
+          <t>Sticker-Zen-0094</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6136,11 +6136,11 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0092</t>
+          <t>Sticker-Zen-0095</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -6155,22 +6155,22 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I106" t="b">
@@ -6186,11 +6186,11 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0093</t>
+          <t>Sticker-Zen-0096</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6205,22 +6205,22 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I107" t="b">
@@ -6236,11 +6236,11 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0094</t>
+          <t>Sticker-Zen-0097</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6255,22 +6255,22 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I108" t="b">
@@ -6290,7 +6290,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0095</t>
+          <t>Sticker-Zen-0098</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0096</t>
+          <t>Sticker-Zen-0099</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0097</t>
+          <t>Sticker-Zen-0100</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0098</t>
+          <t>Sticker-Zen-0101</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0099</t>
+          <t>Sticker-Zen-0102</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0100</t>
+          <t>Sticker-Zen-0103</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0101</t>
+          <t>Sticker-Zen-0104</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0102</t>
+          <t>Sticker-Zen-0105</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0103</t>
+          <t>Sticker-Zen-0106</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0104</t>
+          <t>Sticker-Zen-0107</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0105</t>
+          <t>Sticker-Zen-0108</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0106</t>
+          <t>Sticker-Zen-0109</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0107</t>
+          <t>Sticker-Zen-0110</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0108</t>
+          <t>Sticker-Zen-0111</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0109</t>
+          <t>Sticker-Zen-0112</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0110</t>
+          <t>Sticker-Zen-0113</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7090,7 +7090,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0111</t>
+          <t>Sticker-Zen-0114</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0112</t>
+          <t>Sticker-Zen-0115</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0113</t>
+          <t>Sticker-Zen-0117</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0114</t>
+          <t>Sticker-Zen-0123</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0115</t>
+          <t>Sticker-Zen-0126</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0117</t>
+          <t>Sticker-Zen-0127</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0123</t>
+          <t>Sticker-Zen-0128</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0126</t>
+          <t>Sticker-Zen-0129</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0127</t>
+          <t>Sticker-Zen-0130</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -7540,7 +7540,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0128</t>
+          <t>Sticker-Zen-0131</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0129</t>
+          <t>Sticker-Zen-0132</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0130</t>
+          <t>Sticker-Zen-0133</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0131</t>
+          <t>Sticker-Zen-0134</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0132</t>
+          <t>Sticker-Zen-0135</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7790,7 +7790,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0133</t>
+          <t>Sticker-Zen-0136</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7840,7 +7840,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0134</t>
+          <t>Sticker-Zen-0138</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0135</t>
+          <t>Sticker-Zen-0139</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0136</t>
+          <t>Sticker-Zen-0150</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0138</t>
+          <t>Sticker-Zen-0151</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0139</t>
+          <t>Sticker-Zen-0153</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0150</t>
+          <t>Sticker-Zen-0154</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0151</t>
+          <t>Sticker-Zen-0155</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8190,7 +8190,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0153</t>
+          <t>Sticker-Zen-0156</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0154</t>
+          <t>Sticker-Zen-0157</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0155</t>
+          <t>Sticker-Zen-0158</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0156</t>
+          <t>Sticker-Zen-0159</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0157</t>
+          <t>Sticker-Zen-0160</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -8436,151 +8436,167 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0158</t>
+          <t>Acrylic-Academia-0001</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I152" t="b">
         <v>0</v>
       </c>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>406902588642</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0159</t>
+          <t>Poster-Academia-0026</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I153" t="b">
         <v>0</v>
       </c>
-      <c r="J153" t="inlineStr"/>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>406909164941</t>
+        </is>
+      </c>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0160</t>
+          <t>Poster-Academia-0027</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I154" t="b">
         <v>0</v>
       </c>
-      <c r="J154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>406909216787</t>
+        </is>
+      </c>
       <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -8590,12 +8606,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Acrylic-Academia-0001</t>
+          <t>Poster-Academia-0028</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -8628,14 +8644,10 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>406902588642</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>406909220927</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>True</t>
@@ -8648,7 +8660,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Poster-Academia-0026</t>
+          <t>Poster-Academia-0081</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -8686,10 +8698,14 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>406909164941</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr"/>
+          <t>406902627420</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="L156" t="inlineStr">
         <is>
           <t>True</t>
@@ -8698,167 +8714,163 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Poster-Academia-0027</t>
+          <t>Acrylic-Grimdark-0012</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>No safe action under current weak-network protocol.</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I157" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>406909216787</t>
+          <t>406909148324</t>
         </is>
       </c>
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Poster-Academia-0028</t>
+          <t>Acrylic-Grimdark-0013</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>No safe action under current weak-network protocol.</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>406909220927</t>
+          <t>406909151733</t>
         </is>
       </c>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Poster-Academia-0081</t>
+          <t>Acrylic-Grimdark-0015</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>No safe action under current weak-network protocol.</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I159" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>406902627420</t>
-        </is>
-      </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>406909166683</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -8868,7 +8880,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0012</t>
+          <t>Acrylic-Grimdark-0017</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8906,7 +8918,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>406909148324</t>
+          <t>406909219066</t>
         </is>
       </c>
       <c r="K160" t="inlineStr"/>
@@ -8922,7 +8934,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0013</t>
+          <t>Acrylic-Grimdark-0018</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -8960,7 +8972,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>406909151733</t>
+          <t>406909222169</t>
         </is>
       </c>
       <c r="K161" t="inlineStr"/>
@@ -8976,7 +8988,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0015</t>
+          <t>Acrylic-Grimdark-0021</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -9014,7 +9026,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>406909166683</t>
+          <t>406909225478</t>
         </is>
       </c>
       <c r="K162" t="inlineStr"/>
@@ -9030,7 +9042,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0017</t>
+          <t>Acrylic-Grimdark-0022</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -9068,7 +9080,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>406909219066</t>
+          <t>406909226531</t>
         </is>
       </c>
       <c r="K163" t="inlineStr"/>
@@ -9084,7 +9096,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0018</t>
+          <t>Acrylic-Grimdark-0023</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -9122,7 +9134,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>406909222169</t>
+          <t>406909228840</t>
         </is>
       </c>
       <c r="K164" t="inlineStr"/>
@@ -9138,7 +9150,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0021</t>
+          <t>Acrylic-Grimdark-0024</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -9176,7 +9188,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>406909225478</t>
+          <t>406909231370</t>
         </is>
       </c>
       <c r="K165" t="inlineStr"/>
@@ -9192,7 +9204,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0022</t>
+          <t>Acrylic-Grimdark-0025</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -9230,7 +9242,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>406909226531</t>
+          <t>406909232068</t>
         </is>
       </c>
       <c r="K166" t="inlineStr"/>
@@ -9246,7 +9258,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0023</t>
+          <t>Acrylic-Grimdark-0026</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -9284,7 +9296,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>406909228840</t>
+          <t>406909232951</t>
         </is>
       </c>
       <c r="K167" t="inlineStr"/>
@@ -9300,7 +9312,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0024</t>
+          <t>Acrylic-Grimdark-0028</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -9338,7 +9350,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>406909231370</t>
+          <t>406909234435</t>
         </is>
       </c>
       <c r="K168" t="inlineStr"/>
@@ -9354,7 +9366,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0025</t>
+          <t>Acrylic-Grimdark-0032</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -9392,7 +9404,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>406909232068</t>
+          <t>406909238227</t>
         </is>
       </c>
       <c r="K169" t="inlineStr"/>
@@ -9408,7 +9420,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0026</t>
+          <t>Acrylic-Grimdark-0034</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -9446,7 +9458,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>406909232951</t>
+          <t>406909242546</t>
         </is>
       </c>
       <c r="K170" t="inlineStr"/>
@@ -9462,7 +9474,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0028</t>
+          <t>Acrylic-Grimdark-0036</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -9500,7 +9512,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>406909234435</t>
+          <t>406909244688</t>
         </is>
       </c>
       <c r="K171" t="inlineStr"/>
@@ -9516,7 +9528,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0032</t>
+          <t>Acrylic-Grimdark-0037</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -9554,7 +9566,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>406909238227</t>
+          <t>406909247161</t>
         </is>
       </c>
       <c r="K172" t="inlineStr"/>
@@ -9570,7 +9582,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0034</t>
+          <t>Acrylic-Zen-0004</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -9580,7 +9592,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -9608,10 +9620,14 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>406909242546</t>
-        </is>
-      </c>
-      <c r="K173" t="inlineStr"/>
+          <t>406902888077</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L173" t="inlineStr">
         <is>
           <t>False</t>
@@ -9624,17 +9640,17 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0036</t>
+          <t>Poster-Academia-0001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -9662,10 +9678,14 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>406909244688</t>
-        </is>
-      </c>
-      <c r="K174" t="inlineStr"/>
+          <t>406902584620</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L174" t="inlineStr">
         <is>
           <t>False</t>
@@ -9678,17 +9698,17 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0037</t>
+          <t>Poster-Academia-0001-FIX1</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -9716,7 +9736,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>406909247161</t>
+          <t>406911589289</t>
         </is>
       </c>
       <c r="K175" t="inlineStr"/>
@@ -9732,17 +9752,17 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0004</t>
+          <t>Poster-Academia-0023</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -9770,14 +9790,10 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>406902888077</t>
-        </is>
-      </c>
-      <c r="K176" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>406909147173</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr"/>
       <c r="L176" t="inlineStr">
         <is>
           <t>False</t>
@@ -9790,7 +9806,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Poster-Academia-0001</t>
+          <t>Poster-Academia-0024</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -9828,14 +9844,10 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>406902584620</t>
-        </is>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>406909150037</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr"/>
       <c r="L177" t="inlineStr">
         <is>
           <t>False</t>
@@ -9848,7 +9860,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Poster-Academia-0001-FIX1</t>
+          <t>Poster-Academia-0025</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -9886,7 +9898,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>406911589289</t>
+          <t>406909153504</t>
         </is>
       </c>
       <c r="K178" t="inlineStr"/>
@@ -9902,7 +9914,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Poster-Academia-0023</t>
+          <t>Poster-Academia-0030</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -9940,7 +9952,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>406909147173</t>
+          <t>406909264998</t>
         </is>
       </c>
       <c r="K179" t="inlineStr"/>
@@ -9956,7 +9968,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Poster-Academia-0024</t>
+          <t>Poster-Academia-0031</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -9994,7 +10006,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>406909150037</t>
+          <t>406909266188</t>
         </is>
       </c>
       <c r="K180" t="inlineStr"/>
@@ -10010,7 +10022,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Poster-Academia-0025</t>
+          <t>Poster-Academia-0032</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -10048,7 +10060,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>406909153504</t>
+          <t>406909268494</t>
         </is>
       </c>
       <c r="K181" t="inlineStr"/>
@@ -10064,7 +10076,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Poster-Academia-0030</t>
+          <t>Poster-Academia-0033</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -10102,7 +10114,7 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>406909264998</t>
+          <t>406909269321</t>
         </is>
       </c>
       <c r="K182" t="inlineStr"/>
@@ -10118,7 +10130,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Poster-Academia-0031</t>
+          <t>Poster-Academia-0034</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -10156,7 +10168,7 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>406909266188</t>
+          <t>406909467980</t>
         </is>
       </c>
       <c r="K183" t="inlineStr"/>
@@ -10172,7 +10184,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Poster-Academia-0032</t>
+          <t>Poster-Academia-0035</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -10210,7 +10222,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>406909268494</t>
+          <t>406909471020</t>
         </is>
       </c>
       <c r="K184" t="inlineStr"/>
@@ -10226,7 +10238,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Poster-Academia-0033</t>
+          <t>Poster-Academia-0037</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -10264,7 +10276,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>406909269321</t>
+          <t>406909473606</t>
         </is>
       </c>
       <c r="K185" t="inlineStr"/>
@@ -10280,7 +10292,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Poster-Academia-0034</t>
+          <t>Poster-Academia-0038</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -10318,7 +10330,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>406909467980</t>
+          <t>406910056059</t>
         </is>
       </c>
       <c r="K186" t="inlineStr"/>
@@ -10334,7 +10346,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Poster-Academia-0035</t>
+          <t>Poster-Academia-0039</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -10372,7 +10384,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>406909471020</t>
+          <t>406910057355</t>
         </is>
       </c>
       <c r="K187" t="inlineStr"/>
@@ -10388,7 +10400,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Poster-Academia-0037</t>
+          <t>Poster-Academia-0040</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -10426,7 +10438,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>406909473606</t>
+          <t>406910058626</t>
         </is>
       </c>
       <c r="K188" t="inlineStr"/>
@@ -10442,7 +10454,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Poster-Academia-0038</t>
+          <t>Poster-Academia-0041</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -10480,7 +10492,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>406910056059</t>
+          <t>406910059060</t>
         </is>
       </c>
       <c r="K189" t="inlineStr"/>
@@ -10496,7 +10508,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Poster-Academia-0039</t>
+          <t>Poster-Academia-0042</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -10534,7 +10546,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>406910057355</t>
+          <t>406910060084</t>
         </is>
       </c>
       <c r="K190" t="inlineStr"/>
@@ -10550,7 +10562,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Poster-Academia-0040</t>
+          <t>Poster-Academia-0082</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -10588,10 +10600,14 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>406910058626</t>
-        </is>
-      </c>
-      <c r="K191" t="inlineStr"/>
+          <t>406902648209</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="L191" t="inlineStr">
         <is>
           <t>False</t>
@@ -10604,7 +10620,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Poster-Academia-0041</t>
+          <t>Poster-Academia-0085</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -10642,10 +10658,14 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>406910059060</t>
-        </is>
-      </c>
-      <c r="K192" t="inlineStr"/>
+          <t>406902882943</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L192" t="inlineStr">
         <is>
           <t>False</t>
@@ -10658,7 +10678,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Poster-Academia-0042</t>
+          <t>Poster-Zen-0003</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -10668,7 +10688,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -10694,11 +10714,7 @@
       <c r="I193" t="b">
         <v>1</v>
       </c>
-      <c r="J193" t="inlineStr">
-        <is>
-          <t>406910060084</t>
-        </is>
-      </c>
+      <c r="J193" t="inlineStr"/>
       <c r="K193" t="inlineStr"/>
       <c r="L193" t="inlineStr">
         <is>
@@ -10712,12 +10728,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Poster-Academia-0082</t>
+          <t>Sticker-Academia-0004</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -10750,12 +10766,12 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>406902648209</t>
+          <t>406892408950</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L194" t="inlineStr">
@@ -10770,12 +10786,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Poster-Academia-0085</t>
+          <t>Sticker-Academia-0005</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -10806,16 +10822,8 @@
       <c r="I195" t="b">
         <v>1</v>
       </c>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t>406902882943</t>
-        </is>
-      </c>
-      <c r="K195" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr">
         <is>
           <t>False</t>
@@ -10828,17 +10836,17 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Poster-Zen-0003</t>
+          <t>Sticker-Academia-0005-FIX1</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -10878,7 +10886,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0004</t>
+          <t>Sticker-Academia-0006</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -10914,16 +10922,8 @@
       <c r="I197" t="b">
         <v>1</v>
       </c>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t>406892408950</t>
-        </is>
-      </c>
-      <c r="K197" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr"/>
       <c r="L197" t="inlineStr">
         <is>
           <t>False</t>
@@ -10936,7 +10936,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0005</t>
+          <t>Sticker-Academia-0006-FIX1</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -10972,7 +10972,11 @@
       <c r="I198" t="b">
         <v>1</v>
       </c>
-      <c r="J198" t="inlineStr"/>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>406909095974</t>
+        </is>
+      </c>
       <c r="K198" t="inlineStr"/>
       <c r="L198" t="inlineStr">
         <is>
@@ -10986,7 +10990,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0005-FIX1</t>
+          <t>Sticker-Academia-0007</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -11036,7 +11040,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0006</t>
+          <t>Sticker-Academia-0007-FIX1</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -11072,7 +11076,11 @@
       <c r="I200" t="b">
         <v>1</v>
       </c>
-      <c r="J200" t="inlineStr"/>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>406909097469</t>
+        </is>
+      </c>
       <c r="K200" t="inlineStr"/>
       <c r="L200" t="inlineStr">
         <is>
@@ -11086,7 +11094,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0006-FIX1</t>
+          <t>Sticker-Academia-0008</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -11122,11 +11130,7 @@
       <c r="I201" t="b">
         <v>1</v>
       </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t>406909095974</t>
-        </is>
-      </c>
+      <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr"/>
       <c r="L201" t="inlineStr">
         <is>
@@ -11140,7 +11144,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0007</t>
+          <t>Sticker-Academia-0008-FIX1</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -11176,7 +11180,11 @@
       <c r="I202" t="b">
         <v>1</v>
       </c>
-      <c r="J202" t="inlineStr"/>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>406909100892</t>
+        </is>
+      </c>
       <c r="K202" t="inlineStr"/>
       <c r="L202" t="inlineStr">
         <is>
@@ -11190,7 +11198,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0007-FIX1</t>
+          <t>Sticker-Academia-0009</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -11226,11 +11234,7 @@
       <c r="I203" t="b">
         <v>1</v>
       </c>
-      <c r="J203" t="inlineStr">
-        <is>
-          <t>406909097469</t>
-        </is>
-      </c>
+      <c r="J203" t="inlineStr"/>
       <c r="K203" t="inlineStr"/>
       <c r="L203" t="inlineStr">
         <is>
@@ -11244,7 +11248,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0008</t>
+          <t>Sticker-Academia-0009-FIX1</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -11280,7 +11284,11 @@
       <c r="I204" t="b">
         <v>1</v>
       </c>
-      <c r="J204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>406909114799</t>
+        </is>
+      </c>
       <c r="K204" t="inlineStr"/>
       <c r="L204" t="inlineStr">
         <is>
@@ -11294,7 +11302,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0008-FIX1</t>
+          <t>Sticker-Academia-0010</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -11330,11 +11338,7 @@
       <c r="I205" t="b">
         <v>1</v>
       </c>
-      <c r="J205" t="inlineStr">
-        <is>
-          <t>406909100892</t>
-        </is>
-      </c>
+      <c r="J205" t="inlineStr"/>
       <c r="K205" t="inlineStr"/>
       <c r="L205" t="inlineStr">
         <is>
@@ -11348,7 +11352,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0009</t>
+          <t>Sticker-Academia-0010-FIX1</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -11384,7 +11388,11 @@
       <c r="I206" t="b">
         <v>1</v>
       </c>
-      <c r="J206" t="inlineStr"/>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>406909116716</t>
+        </is>
+      </c>
       <c r="K206" t="inlineStr"/>
       <c r="L206" t="inlineStr">
         <is>
@@ -11398,7 +11406,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0009-FIX1</t>
+          <t>Sticker-Academia-0011</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -11434,11 +11442,7 @@
       <c r="I207" t="b">
         <v>1</v>
       </c>
-      <c r="J207" t="inlineStr">
-        <is>
-          <t>406909114799</t>
-        </is>
-      </c>
+      <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr"/>
       <c r="L207" t="inlineStr">
         <is>
@@ -11452,7 +11456,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0010</t>
+          <t>Sticker-Academia-0011-FIX1</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -11488,7 +11492,11 @@
       <c r="I208" t="b">
         <v>1</v>
       </c>
-      <c r="J208" t="inlineStr"/>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>406909118000</t>
+        </is>
+      </c>
       <c r="K208" t="inlineStr"/>
       <c r="L208" t="inlineStr">
         <is>
@@ -11502,7 +11510,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0010-FIX1</t>
+          <t>Sticker-Academia-0014</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -11538,11 +11546,7 @@
       <c r="I209" t="b">
         <v>1</v>
       </c>
-      <c r="J209" t="inlineStr">
-        <is>
-          <t>406909116716</t>
-        </is>
-      </c>
+      <c r="J209" t="inlineStr"/>
       <c r="K209" t="inlineStr"/>
       <c r="L209" t="inlineStr">
         <is>
@@ -11556,7 +11560,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0011</t>
+          <t>Sticker-Academia-0014-FIX1</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -11592,7 +11596,11 @@
       <c r="I210" t="b">
         <v>1</v>
       </c>
-      <c r="J210" t="inlineStr"/>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>406909119544</t>
+        </is>
+      </c>
       <c r="K210" t="inlineStr"/>
       <c r="L210" t="inlineStr">
         <is>
@@ -11606,7 +11614,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0011-FIX1</t>
+          <t>Sticker-Academia-0015</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -11642,11 +11650,7 @@
       <c r="I211" t="b">
         <v>1</v>
       </c>
-      <c r="J211" t="inlineStr">
-        <is>
-          <t>406909118000</t>
-        </is>
-      </c>
+      <c r="J211" t="inlineStr"/>
       <c r="K211" t="inlineStr"/>
       <c r="L211" t="inlineStr">
         <is>
@@ -11660,7 +11664,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0014</t>
+          <t>Sticker-Academia-0015-FIX1</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -11696,7 +11700,11 @@
       <c r="I212" t="b">
         <v>1</v>
       </c>
-      <c r="J212" t="inlineStr"/>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>406909121336</t>
+        </is>
+      </c>
       <c r="K212" t="inlineStr"/>
       <c r="L212" t="inlineStr">
         <is>
@@ -11710,7 +11718,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0014-FIX1</t>
+          <t>Sticker-Academia-0016</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -11746,11 +11754,7 @@
       <c r="I213" t="b">
         <v>1</v>
       </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>406909119544</t>
-        </is>
-      </c>
+      <c r="J213" t="inlineStr"/>
       <c r="K213" t="inlineStr"/>
       <c r="L213" t="inlineStr">
         <is>
@@ -11764,7 +11768,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0015</t>
+          <t>Sticker-Academia-0016-FIX1</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -11800,7 +11804,11 @@
       <c r="I214" t="b">
         <v>1</v>
       </c>
-      <c r="J214" t="inlineStr"/>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>406909122790</t>
+        </is>
+      </c>
       <c r="K214" t="inlineStr"/>
       <c r="L214" t="inlineStr">
         <is>
@@ -11814,7 +11822,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0015-FIX1</t>
+          <t>Sticker-Zen-0001</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -11824,7 +11832,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -11850,11 +11858,7 @@
       <c r="I215" t="b">
         <v>1</v>
       </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t>406909121336</t>
-        </is>
-      </c>
+      <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr"/>
       <c r="L215" t="inlineStr">
         <is>
@@ -11868,7 +11872,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0016</t>
+          <t>Sticker-Zen-0001-FIX1</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -11878,7 +11882,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -11904,7 +11908,11 @@
       <c r="I216" t="b">
         <v>1</v>
       </c>
-      <c r="J216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>406909124585</t>
+        </is>
+      </c>
       <c r="K216" t="inlineStr"/>
       <c r="L216" t="inlineStr">
         <is>
@@ -11918,7 +11926,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0016-FIX1</t>
+          <t>Sticker-Zen-0002</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -11928,7 +11936,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -11954,11 +11962,7 @@
       <c r="I217" t="b">
         <v>1</v>
       </c>
-      <c r="J217" t="inlineStr">
-        <is>
-          <t>406909122790</t>
-        </is>
-      </c>
+      <c r="J217" t="inlineStr"/>
       <c r="K217" t="inlineStr"/>
       <c r="L217" t="inlineStr">
         <is>
@@ -11972,7 +11976,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0001</t>
+          <t>Sticker-Zen-0002-FIX1</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -12008,7 +12012,11 @@
       <c r="I218" t="b">
         <v>1</v>
       </c>
-      <c r="J218" t="inlineStr"/>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>406909125700</t>
+        </is>
+      </c>
       <c r="K218" t="inlineStr"/>
       <c r="L218" t="inlineStr">
         <is>
@@ -12022,7 +12030,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0001-FIX1</t>
+          <t>Sticker-Zen-0003</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -12058,11 +12066,7 @@
       <c r="I219" t="b">
         <v>1</v>
       </c>
-      <c r="J219" t="inlineStr">
-        <is>
-          <t>406909124585</t>
-        </is>
-      </c>
+      <c r="J219" t="inlineStr"/>
       <c r="K219" t="inlineStr"/>
       <c r="L219" t="inlineStr">
         <is>
@@ -12076,7 +12080,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0002</t>
+          <t>Sticker-Zen-0003-FIX1</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -12112,7 +12116,11 @@
       <c r="I220" t="b">
         <v>1</v>
       </c>
-      <c r="J220" t="inlineStr"/>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>406909126789</t>
+        </is>
+      </c>
       <c r="K220" t="inlineStr"/>
       <c r="L220" t="inlineStr">
         <is>
@@ -12126,7 +12134,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0002-FIX1</t>
+          <t>Sticker-Zen-0004</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -12162,11 +12170,7 @@
       <c r="I221" t="b">
         <v>1</v>
       </c>
-      <c r="J221" t="inlineStr">
-        <is>
-          <t>406909125700</t>
-        </is>
-      </c>
+      <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr"/>
       <c r="L221" t="inlineStr">
         <is>
@@ -12180,7 +12184,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0003</t>
+          <t>Sticker-Zen-0004-FIX1</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -12216,7 +12220,11 @@
       <c r="I222" t="b">
         <v>1</v>
       </c>
-      <c r="J222" t="inlineStr"/>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>406909127704</t>
+        </is>
+      </c>
       <c r="K222" t="inlineStr"/>
       <c r="L222" t="inlineStr">
         <is>
@@ -12230,7 +12238,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0003-FIX1</t>
+          <t>Sticker-Zen-0005</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -12266,11 +12274,7 @@
       <c r="I223" t="b">
         <v>1</v>
       </c>
-      <c r="J223" t="inlineStr">
-        <is>
-          <t>406909126789</t>
-        </is>
-      </c>
+      <c r="J223" t="inlineStr"/>
       <c r="K223" t="inlineStr"/>
       <c r="L223" t="inlineStr">
         <is>
@@ -12284,7 +12288,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0004</t>
+          <t>Sticker-Zen-0005-FIX1</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -12320,7 +12324,11 @@
       <c r="I224" t="b">
         <v>1</v>
       </c>
-      <c r="J224" t="inlineStr"/>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>406909342825</t>
+        </is>
+      </c>
       <c r="K224" t="inlineStr"/>
       <c r="L224" t="inlineStr">
         <is>
@@ -12334,7 +12342,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0004-FIX1</t>
+          <t>Sticker-Zen-0007</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -12370,11 +12378,7 @@
       <c r="I225" t="b">
         <v>1</v>
       </c>
-      <c r="J225" t="inlineStr">
-        <is>
-          <t>406909127704</t>
-        </is>
-      </c>
+      <c r="J225" t="inlineStr"/>
       <c r="K225" t="inlineStr"/>
       <c r="L225" t="inlineStr">
         <is>
@@ -12388,7 +12392,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0005</t>
+          <t>Sticker-Zen-0007-FIX1</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -12424,7 +12428,11 @@
       <c r="I226" t="b">
         <v>1</v>
       </c>
-      <c r="J226" t="inlineStr"/>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>406909344491</t>
+        </is>
+      </c>
       <c r="K226" t="inlineStr"/>
       <c r="L226" t="inlineStr">
         <is>
@@ -12438,7 +12446,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0005-FIX1</t>
+          <t>Sticker-Zen-0008</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -12474,11 +12482,7 @@
       <c r="I227" t="b">
         <v>1</v>
       </c>
-      <c r="J227" t="inlineStr">
-        <is>
-          <t>406909342825</t>
-        </is>
-      </c>
+      <c r="J227" t="inlineStr"/>
       <c r="K227" t="inlineStr"/>
       <c r="L227" t="inlineStr">
         <is>
@@ -12492,7 +12496,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0007</t>
+          <t>Sticker-Zen-0008-FIX1</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -12528,7 +12532,11 @@
       <c r="I228" t="b">
         <v>1</v>
       </c>
-      <c r="J228" t="inlineStr"/>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>406909345291</t>
+        </is>
+      </c>
       <c r="K228" t="inlineStr"/>
       <c r="L228" t="inlineStr">
         <is>
@@ -12542,7 +12550,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0007-FIX1</t>
+          <t>Sticker-Zen-0009</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -12578,11 +12586,7 @@
       <c r="I229" t="b">
         <v>1</v>
       </c>
-      <c r="J229" t="inlineStr">
-        <is>
-          <t>406909344491</t>
-        </is>
-      </c>
+      <c r="J229" t="inlineStr"/>
       <c r="K229" t="inlineStr"/>
       <c r="L229" t="inlineStr">
         <is>
@@ -12596,7 +12600,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0008</t>
+          <t>Sticker-Zen-0009-FIX1</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -12632,7 +12636,11 @@
       <c r="I230" t="b">
         <v>1</v>
       </c>
-      <c r="J230" t="inlineStr"/>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>406909353931</t>
+        </is>
+      </c>
       <c r="K230" t="inlineStr"/>
       <c r="L230" t="inlineStr">
         <is>
@@ -12646,7 +12654,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0008-FIX1</t>
+          <t>Sticker-Zen-0022</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -12682,11 +12690,7 @@
       <c r="I231" t="b">
         <v>1</v>
       </c>
-      <c r="J231" t="inlineStr">
-        <is>
-          <t>406909345291</t>
-        </is>
-      </c>
+      <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr">
         <is>
@@ -12700,7 +12704,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0009</t>
+          <t>Sticker-Zen-0022-FIX1</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -12736,7 +12740,11 @@
       <c r="I232" t="b">
         <v>1</v>
       </c>
-      <c r="J232" t="inlineStr"/>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>406909354903</t>
+        </is>
+      </c>
       <c r="K232" t="inlineStr"/>
       <c r="L232" t="inlineStr">
         <is>
@@ -12750,7 +12758,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0009-FIX1</t>
+          <t>Sticker-Zen-0024</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -12786,11 +12794,7 @@
       <c r="I233" t="b">
         <v>1</v>
       </c>
-      <c r="J233" t="inlineStr">
-        <is>
-          <t>406909353931</t>
-        </is>
-      </c>
+      <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr"/>
       <c r="L233" t="inlineStr">
         <is>
@@ -12804,7 +12808,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0022</t>
+          <t>Sticker-Zen-0024-FIX1</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -12840,7 +12844,11 @@
       <c r="I234" t="b">
         <v>1</v>
       </c>
-      <c r="J234" t="inlineStr"/>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>406909355853</t>
+        </is>
+      </c>
       <c r="K234" t="inlineStr"/>
       <c r="L234" t="inlineStr">
         <is>
@@ -12854,7 +12862,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0022-FIX1</t>
+          <t>Sticker-Zen-0025</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -12890,11 +12898,7 @@
       <c r="I235" t="b">
         <v>1</v>
       </c>
-      <c r="J235" t="inlineStr">
-        <is>
-          <t>406909354903</t>
-        </is>
-      </c>
+      <c r="J235" t="inlineStr"/>
       <c r="K235" t="inlineStr"/>
       <c r="L235" t="inlineStr">
         <is>
@@ -12908,7 +12912,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0024</t>
+          <t>Sticker-Zen-0025-FIX1</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -12944,7 +12948,11 @@
       <c r="I236" t="b">
         <v>1</v>
       </c>
-      <c r="J236" t="inlineStr"/>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>406909359949</t>
+        </is>
+      </c>
       <c r="K236" t="inlineStr"/>
       <c r="L236" t="inlineStr">
         <is>
@@ -12958,7 +12966,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0024-FIX1</t>
+          <t>Sticker-Zen-0026</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -12994,11 +13002,7 @@
       <c r="I237" t="b">
         <v>1</v>
       </c>
-      <c r="J237" t="inlineStr">
-        <is>
-          <t>406909355853</t>
-        </is>
-      </c>
+      <c r="J237" t="inlineStr"/>
       <c r="K237" t="inlineStr"/>
       <c r="L237" t="inlineStr">
         <is>
@@ -13012,7 +13016,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0025</t>
+          <t>Sticker-Zen-0027</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -13062,7 +13066,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0025-FIX1</t>
+          <t>Sticker-Zen-0027-FIX1</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -13100,7 +13104,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>406909359949</t>
+          <t>406909364977</t>
         </is>
       </c>
       <c r="K239" t="inlineStr"/>
@@ -13116,7 +13120,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0026</t>
+          <t>Sticker-Zen-0029</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -13166,7 +13170,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0027</t>
+          <t>Sticker-Zen-0031</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -13216,7 +13220,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0027-FIX1</t>
+          <t>Sticker-Zen-0032</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -13252,11 +13256,7 @@
       <c r="I242" t="b">
         <v>1</v>
       </c>
-      <c r="J242" t="inlineStr">
-        <is>
-          <t>406909364977</t>
-        </is>
-      </c>
+      <c r="J242" t="inlineStr"/>
       <c r="K242" t="inlineStr"/>
       <c r="L242" t="inlineStr">
         <is>
@@ -13270,7 +13270,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0029</t>
+          <t>Sticker-Zen-0034</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0031</t>
+          <t>Sticker-Zen-0035</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -13370,7 +13370,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0032</t>
+          <t>Sticker-Zen-0036</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -13420,7 +13420,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0034</t>
+          <t>Sticker-Zen-0037</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -13470,7 +13470,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0035</t>
+          <t>Sticker-Zen-0038</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0036</t>
+          <t>Sticker-Zen-0040</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0037</t>
+          <t>Sticker-Zen-0041</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -13620,7 +13620,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0038</t>
+          <t>Sticker-Zen-0041-FIX1</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -13656,7 +13656,11 @@
       <c r="I250" t="b">
         <v>1</v>
       </c>
-      <c r="J250" t="inlineStr"/>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>406909368739</t>
+        </is>
+      </c>
       <c r="K250" t="inlineStr"/>
       <c r="L250" t="inlineStr">
         <is>
@@ -13670,7 +13674,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0040</t>
+          <t>Sticker-Zen-0042</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -13720,7 +13724,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0041</t>
+          <t>Sticker-Zen-0042-FIX1</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -13756,7 +13760,11 @@
       <c r="I252" t="b">
         <v>1</v>
       </c>
-      <c r="J252" t="inlineStr"/>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>406909373586</t>
+        </is>
+      </c>
       <c r="K252" t="inlineStr"/>
       <c r="L252" t="inlineStr">
         <is>
@@ -13770,7 +13778,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0041-FIX1</t>
+          <t>Sticker-Zen-0044</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -13808,10 +13816,14 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>406909368739</t>
-        </is>
-      </c>
-      <c r="K253" t="inlineStr"/>
+          <t>406902622710</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L253" t="inlineStr">
         <is>
           <t>False</t>
@@ -13824,7 +13836,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0042</t>
+          <t>Sticker-Zen-0044-FIX1</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -13860,7 +13872,11 @@
       <c r="I254" t="b">
         <v>1</v>
       </c>
-      <c r="J254" t="inlineStr"/>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>406909884756</t>
+        </is>
+      </c>
       <c r="K254" t="inlineStr"/>
       <c r="L254" t="inlineStr">
         <is>
@@ -13874,7 +13890,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0042-FIX1</t>
+          <t>Sticker-Zen-0045</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -13912,10 +13928,14 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>406909373586</t>
-        </is>
-      </c>
-      <c r="K255" t="inlineStr"/>
+          <t>406902640998</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L255" t="inlineStr">
         <is>
           <t>False</t>
@@ -13928,7 +13948,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0044</t>
+          <t>Sticker-Zen-0045-FIX1</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -13966,14 +13986,10 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>406902622710</t>
-        </is>
-      </c>
-      <c r="K256" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909890800</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr"/>
       <c r="L256" t="inlineStr">
         <is>
           <t>False</t>
@@ -13986,7 +14002,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0044-FIX1</t>
+          <t>Sticker-Zen-0046</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -14024,10 +14040,14 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>406909884756</t>
-        </is>
-      </c>
-      <c r="K257" t="inlineStr"/>
+          <t>406902663232</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L257" t="inlineStr">
         <is>
           <t>False</t>
@@ -14040,7 +14060,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0045</t>
+          <t>Sticker-Zen-0046-FIX1</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -14078,14 +14098,10 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>406902640998</t>
-        </is>
-      </c>
-      <c r="K258" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909891985</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr"/>
       <c r="L258" t="inlineStr">
         <is>
           <t>False</t>
@@ -14098,7 +14114,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0045-FIX1</t>
+          <t>Sticker-Zen-0048</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -14134,11 +14150,7 @@
       <c r="I259" t="b">
         <v>1</v>
       </c>
-      <c r="J259" t="inlineStr">
-        <is>
-          <t>406909890800</t>
-        </is>
-      </c>
+      <c r="J259" t="inlineStr"/>
       <c r="K259" t="inlineStr"/>
       <c r="L259" t="inlineStr">
         <is>
@@ -14152,7 +14164,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0046</t>
+          <t>Sticker-Zen-0049</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -14190,7 +14202,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>406902663232</t>
+          <t>406902713267</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -14210,7 +14222,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0046-FIX1</t>
+          <t>Sticker-Zen-0049-FIX1</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -14248,7 +14260,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>406909891985</t>
+          <t>406909893702</t>
         </is>
       </c>
       <c r="K261" t="inlineStr"/>
@@ -14264,7 +14276,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0048</t>
+          <t>Sticker-Zen-0050</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -14300,8 +14312,16 @@
       <c r="I262" t="b">
         <v>1</v>
       </c>
-      <c r="J262" t="inlineStr"/>
-      <c r="K262" t="inlineStr"/>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>406902886081</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L262" t="inlineStr">
         <is>
           <t>False</t>
@@ -14314,7 +14334,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0049</t>
+          <t>Sticker-Zen-0050-FIX1</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -14352,14 +14372,10 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>406902713267</t>
-        </is>
-      </c>
-      <c r="K263" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909904704</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr"/>
       <c r="L263" t="inlineStr">
         <is>
           <t>False</t>
@@ -14372,7 +14388,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0049-FIX1</t>
+          <t>Sticker-Zen-0051</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -14410,10 +14426,14 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>406909893702</t>
-        </is>
-      </c>
-      <c r="K264" t="inlineStr"/>
+          <t>406902889638</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L264" t="inlineStr">
         <is>
           <t>False</t>
@@ -14426,7 +14446,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0050</t>
+          <t>Sticker-Zen-0051-FIX1</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -14464,14 +14484,10 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>406902886081</t>
-        </is>
-      </c>
-      <c r="K265" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909905683</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr"/>
       <c r="L265" t="inlineStr">
         <is>
           <t>False</t>
@@ -14484,7 +14500,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0050-FIX1</t>
+          <t>Sticker-Zen-0052</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -14522,10 +14538,14 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>406909904704</t>
-        </is>
-      </c>
-      <c r="K266" t="inlineStr"/>
+          <t>406902896387</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L266" t="inlineStr">
         <is>
           <t>False</t>
@@ -14538,7 +14558,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0051</t>
+          <t>Sticker-Zen-0052-FIX1</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -14576,14 +14596,10 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>406902889638</t>
-        </is>
-      </c>
-      <c r="K267" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909906686</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr"/>
       <c r="L267" t="inlineStr">
         <is>
           <t>False</t>
@@ -14596,7 +14612,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0051-FIX1</t>
+          <t>Sticker-Zen-0053</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -14634,10 +14650,14 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>406909905683</t>
-        </is>
-      </c>
-      <c r="K268" t="inlineStr"/>
+          <t>406902900109</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L268" t="inlineStr">
         <is>
           <t>False</t>
@@ -14650,7 +14670,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0052</t>
+          <t>Sticker-Zen-0053-FIX1</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -14688,14 +14708,10 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>406902896387</t>
-        </is>
-      </c>
-      <c r="K269" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909907111</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr"/>
       <c r="L269" t="inlineStr">
         <is>
           <t>False</t>
@@ -14708,7 +14724,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0052-FIX1</t>
+          <t>Sticker-Zen-0054</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -14746,10 +14762,14 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>406909906686</t>
-        </is>
-      </c>
-      <c r="K270" t="inlineStr"/>
+          <t>406903032635</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L270" t="inlineStr">
         <is>
           <t>False</t>
@@ -14762,7 +14782,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0053</t>
+          <t>Sticker-Zen-0054-FIX1</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -14800,14 +14820,10 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>406902900109</t>
-        </is>
-      </c>
-      <c r="K271" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909907742</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr"/>
       <c r="L271" t="inlineStr">
         <is>
           <t>False</t>
@@ -14820,7 +14836,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0053-FIX1</t>
+          <t>Sticker-Zen-0055</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -14858,10 +14874,14 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>406909907111</t>
-        </is>
-      </c>
-      <c r="K272" t="inlineStr"/>
+          <t>406903037933</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L272" t="inlineStr">
         <is>
           <t>False</t>
@@ -14874,7 +14894,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0054</t>
+          <t>Sticker-Zen-0055-FIX1</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -14912,14 +14932,10 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>406903032635</t>
-        </is>
-      </c>
-      <c r="K273" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406910984204</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr"/>
       <c r="L273" t="inlineStr">
         <is>
           <t>False</t>
@@ -14932,7 +14948,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0054-FIX1</t>
+          <t>Sticker-Zen-0056</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -14970,10 +14986,14 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>406909907742</t>
-        </is>
-      </c>
-      <c r="K274" t="inlineStr"/>
+          <t>406903041315</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L274" t="inlineStr">
         <is>
           <t>False</t>
@@ -14986,7 +15006,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0055</t>
+          <t>Sticker-Zen-0056-FIX1</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -15024,14 +15044,10 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>406903037933</t>
-        </is>
-      </c>
-      <c r="K275" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911030956</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr"/>
       <c r="L275" t="inlineStr">
         <is>
           <t>False</t>
@@ -15044,7 +15060,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0055-FIX1</t>
+          <t>Sticker-Zen-0057</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -15082,10 +15098,14 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>406910984204</t>
-        </is>
-      </c>
-      <c r="K276" t="inlineStr"/>
+          <t>406903044643</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L276" t="inlineStr">
         <is>
           <t>False</t>
@@ -15098,7 +15118,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0056</t>
+          <t>Sticker-Zen-0057-FIX1</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -15136,14 +15156,10 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>406903041315</t>
-        </is>
-      </c>
-      <c r="K277" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911046712</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr"/>
       <c r="L277" t="inlineStr">
         <is>
           <t>False</t>
@@ -15156,7 +15172,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0056-FIX1</t>
+          <t>Sticker-Zen-0058</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -15194,10 +15210,14 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>406911030956</t>
-        </is>
-      </c>
-      <c r="K278" t="inlineStr"/>
+          <t>406903049411</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L278" t="inlineStr">
         <is>
           <t>False</t>
@@ -15210,7 +15230,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0057</t>
+          <t>Sticker-Zen-0058-FIX1</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -15248,14 +15268,10 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>406903044643</t>
-        </is>
-      </c>
-      <c r="K279" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911102240</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr"/>
       <c r="L279" t="inlineStr">
         <is>
           <t>False</t>
@@ -15268,7 +15284,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0057-FIX1</t>
+          <t>Sticker-Zen-0060</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -15306,10 +15322,14 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>406911046712</t>
-        </is>
-      </c>
-      <c r="K280" t="inlineStr"/>
+          <t>406903249053</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L280" t="inlineStr">
         <is>
           <t>False</t>
@@ -15322,7 +15342,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0058</t>
+          <t>Sticker-Zen-0060-FIX1</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -15360,14 +15380,10 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>406903049411</t>
-        </is>
-      </c>
-      <c r="K281" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911120974</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr"/>
       <c r="L281" t="inlineStr">
         <is>
           <t>False</t>
@@ -15380,7 +15396,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0058-FIX1</t>
+          <t>Sticker-Zen-0061</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -15418,10 +15434,14 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>406911102240</t>
-        </is>
-      </c>
-      <c r="K282" t="inlineStr"/>
+          <t>406903249987</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L282" t="inlineStr">
         <is>
           <t>False</t>
@@ -15434,7 +15454,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0060</t>
+          <t>Sticker-Zen-0061-FIX1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -15472,14 +15492,10 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>406903249053</t>
-        </is>
-      </c>
-      <c r="K283" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911452547</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr"/>
       <c r="L283" t="inlineStr">
         <is>
           <t>False</t>
@@ -15492,7 +15508,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0060-FIX1</t>
+          <t>Sticker-Zen-0062</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -15530,10 +15546,14 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>406911120974</t>
-        </is>
-      </c>
-      <c r="K284" t="inlineStr"/>
+          <t>406903250891</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L284" t="inlineStr">
         <is>
           <t>False</t>
@@ -15546,7 +15566,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0061</t>
+          <t>Sticker-Zen-0062-FIX1</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -15584,14 +15604,10 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>406903249987</t>
-        </is>
-      </c>
-      <c r="K285" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911488570</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr"/>
       <c r="L285" t="inlineStr">
         <is>
           <t>False</t>
@@ -15604,7 +15620,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0061-FIX1</t>
+          <t>Sticker-Zen-0063</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -15642,10 +15658,14 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>406911452547</t>
-        </is>
-      </c>
-      <c r="K286" t="inlineStr"/>
+          <t>406903252007</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L286" t="inlineStr">
         <is>
           <t>False</t>
@@ -15658,7 +15678,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0062</t>
+          <t>Sticker-Zen-0063-FIX1</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -15696,14 +15716,10 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>406903250891</t>
-        </is>
-      </c>
-      <c r="K287" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911494155</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr"/>
       <c r="L287" t="inlineStr">
         <is>
           <t>False</t>
@@ -15716,7 +15732,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0062-FIX1</t>
+          <t>Sticker-Zen-0066</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -15754,7 +15770,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>406911488570</t>
+          <t>406903252739</t>
         </is>
       </c>
       <c r="K288" t="inlineStr"/>
@@ -15770,7 +15786,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0063</t>
+          <t>Sticker-Zen-0066-FIX1</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -15808,14 +15824,10 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>406903252007</t>
-        </is>
-      </c>
-      <c r="K289" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911509730</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr"/>
       <c r="L289" t="inlineStr">
         <is>
           <t>False</t>
@@ -15828,7 +15840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0063-FIX1</t>
+          <t>Sticker-Zen-0067</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -15864,11 +15876,7 @@
       <c r="I290" t="b">
         <v>1</v>
       </c>
-      <c r="J290" t="inlineStr">
-        <is>
-          <t>406911494155</t>
-        </is>
-      </c>
+      <c r="J290" t="inlineStr"/>
       <c r="K290" t="inlineStr"/>
       <c r="L290" t="inlineStr">
         <is>
@@ -15882,7 +15890,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0066</t>
+          <t>Sticker-Zen-0068</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -15918,11 +15926,7 @@
       <c r="I291" t="b">
         <v>1</v>
       </c>
-      <c r="J291" t="inlineStr">
-        <is>
-          <t>406903252739</t>
-        </is>
-      </c>
+      <c r="J291" t="inlineStr"/>
       <c r="K291" t="inlineStr"/>
       <c r="L291" t="inlineStr">
         <is>
@@ -15936,7 +15940,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0066-FIX1</t>
+          <t>Sticker-Zen-0069</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -15974,7 +15978,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>406911509730</t>
+          <t>406903753067</t>
         </is>
       </c>
       <c r="K292" t="inlineStr"/>
@@ -15990,7 +15994,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0067</t>
+          <t>Sticker-Zen-0069-FIX1</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -16026,7 +16030,11 @@
       <c r="I293" t="b">
         <v>1</v>
       </c>
-      <c r="J293" t="inlineStr"/>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>406911531255</t>
+        </is>
+      </c>
       <c r="K293" t="inlineStr"/>
       <c r="L293" t="inlineStr">
         <is>
@@ -16040,7 +16048,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0068</t>
+          <t>Sticker-Zen-0070</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -16076,7 +16084,11 @@
       <c r="I294" t="b">
         <v>1</v>
       </c>
-      <c r="J294" t="inlineStr"/>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>406903757240</t>
+        </is>
+      </c>
       <c r="K294" t="inlineStr"/>
       <c r="L294" t="inlineStr">
         <is>
@@ -16090,7 +16102,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0069</t>
+          <t>Sticker-Zen-0070-FIX1</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -16128,7 +16140,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>406903753067</t>
+          <t>406911541926</t>
         </is>
       </c>
       <c r="K295" t="inlineStr"/>
@@ -16144,7 +16156,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0069-FIX1</t>
+          <t>Sticker-Zen-0071</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -16182,7 +16194,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>406911531255</t>
+          <t>406903762328</t>
         </is>
       </c>
       <c r="K296" t="inlineStr"/>
@@ -16198,7 +16210,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0070</t>
+          <t>Sticker-Zen-0071-FIX1</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -16236,7 +16248,7 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>406903757240</t>
+          <t>406911551031</t>
         </is>
       </c>
       <c r="K297" t="inlineStr"/>
@@ -16252,7 +16264,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0070-FIX1</t>
+          <t>Sticker-Zen-0072</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -16290,7 +16302,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>406911541926</t>
+          <t>406911942577</t>
         </is>
       </c>
       <c r="K298" t="inlineStr"/>
@@ -16306,7 +16318,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0071</t>
+          <t>Sticker-Zen-0073</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -16344,7 +16356,7 @@
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>406903762328</t>
+          <t>406911955913</t>
         </is>
       </c>
       <c r="K299" t="inlineStr"/>
@@ -16360,7 +16372,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0071-FIX1</t>
+          <t>Sticker-Zen-0074</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -16398,7 +16410,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>406911551031</t>
+          <t>406911953636</t>
         </is>
       </c>
       <c r="K300" t="inlineStr"/>

</xml_diff>

<commit_message>
Harden sticker gallery workflow and refresh queues
</commit_message>
<xml_diff>
--- a/Database/Market_Signal_Action_Queue.xlsx
+++ b/Database/Market_Signal_Action_Queue.xlsx
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0075</t>
+          <t>Sticker-Zen-0083</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0076</t>
+          <t>Sticker-Zen-0084</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0081</t>
+          <t>Sticker-Zen-0086</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0083</t>
+          <t>Sticker-Zen-0087</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0084</t>
+          <t>Sticker-Zen-0088</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0086</t>
+          <t>Sticker-Zen-0089</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0087</t>
+          <t>Sticker-Zen-0091</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0088</t>
+          <t>Sticker-Zen-0092</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0089</t>
+          <t>Sticker-Zen-0093</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0091</t>
+          <t>Sticker-Zen-0094</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5986,11 +5986,11 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0092</t>
+          <t>Sticker-Zen-0095</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6005,22 +6005,22 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I103" t="b">
@@ -6036,11 +6036,11 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0093</t>
+          <t>Sticker-Zen-0096</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6055,22 +6055,22 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I104" t="b">
@@ -6086,11 +6086,11 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0094</t>
+          <t>Sticker-Zen-0097</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6105,22 +6105,22 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Stable_Draft_Publish_When_Scheduled</t>
+          <t>Ready_For_Printify_When_Network_OK</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>PUBLISH_IN_SMALL_BATCH_WHEN_NETWORK_OK</t>
+          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Stable Printify mockups exist; publish only via cooled scheduler and audit image order afterward.</t>
+          <t>Local assets are ready but network-dependent upload remains pending.</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I105" t="b">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0095</t>
+          <t>Sticker-Zen-0098</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0096</t>
+          <t>Sticker-Zen-0099</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0097</t>
+          <t>Sticker-Zen-0100</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6290,7 +6290,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0098</t>
+          <t>Sticker-Zen-0101</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0099</t>
+          <t>Sticker-Zen-0102</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0100</t>
+          <t>Sticker-Zen-0103</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0101</t>
+          <t>Sticker-Zen-0104</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0102</t>
+          <t>Sticker-Zen-0105</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0103</t>
+          <t>Sticker-Zen-0106</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0104</t>
+          <t>Sticker-Zen-0107</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0105</t>
+          <t>Sticker-Zen-0108</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0106</t>
+          <t>Sticker-Zen-0109</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0107</t>
+          <t>Sticker-Zen-0110</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0108</t>
+          <t>Sticker-Zen-0111</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0109</t>
+          <t>Sticker-Zen-0112</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0110</t>
+          <t>Sticker-Zen-0113</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0111</t>
+          <t>Sticker-Zen-0114</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0112</t>
+          <t>Sticker-Zen-0115</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0113</t>
+          <t>Sticker-Zen-0117</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7090,7 +7090,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0114</t>
+          <t>Sticker-Zen-0123</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0115</t>
+          <t>Sticker-Zen-0126</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0117</t>
+          <t>Sticker-Zen-0127</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0123</t>
+          <t>Sticker-Zen-0128</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0126</t>
+          <t>Sticker-Zen-0129</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0127</t>
+          <t>Sticker-Zen-0130</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0128</t>
+          <t>Sticker-Zen-0131</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0129</t>
+          <t>Sticker-Zen-0132</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0130</t>
+          <t>Sticker-Zen-0133</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -7540,7 +7540,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0131</t>
+          <t>Sticker-Zen-0134</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0132</t>
+          <t>Sticker-Zen-0135</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0133</t>
+          <t>Sticker-Zen-0136</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0134</t>
+          <t>Sticker-Zen-0138</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0135</t>
+          <t>Sticker-Zen-0139</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7790,7 +7790,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0136</t>
+          <t>Sticker-Zen-0150</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7840,7 +7840,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0138</t>
+          <t>Sticker-Zen-0151</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0139</t>
+          <t>Sticker-Zen-0153</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0150</t>
+          <t>Sticker-Zen-0154</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0151</t>
+          <t>Sticker-Zen-0155</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0153</t>
+          <t>Sticker-Zen-0156</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0154</t>
+          <t>Sticker-Zen-0157</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0155</t>
+          <t>Sticker-Zen-0158</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8190,7 +8190,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0156</t>
+          <t>Sticker-Zen-0159</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0157</t>
+          <t>Sticker-Zen-0160</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -8286,151 +8286,167 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0158</t>
+          <t>Acrylic-Academia-0001</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I149" t="b">
         <v>0</v>
       </c>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>406902588642</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0159</t>
+          <t>Poster-Academia-0026</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I150" t="b">
         <v>0</v>
       </c>
-      <c r="J150" t="inlineStr"/>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>406909164941</t>
+        </is>
+      </c>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0160</t>
+          <t>Poster-Academia-0027</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Ready_For_Printify_When_Network_OK</t>
+          <t>Etsy_Draft_Prepared</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>UPLOAD_TO_PRINTIFY_SINGLE_ITEM_BATCH</t>
+          <t>KEEP_FOR_ETSY_PHASE1</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Local assets are ready but network-dependent upload remains pending.</t>
+          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I151" t="b">
         <v>0</v>
       </c>
-      <c r="J151" t="inlineStr"/>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>406909216787</t>
+        </is>
+      </c>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -8440,12 +8456,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Acrylic-Academia-0001</t>
+          <t>Poster-Academia-0028</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -8478,14 +8494,10 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>406902588642</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>406909220927</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr">
         <is>
           <t>True</t>
@@ -8498,7 +8510,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Poster-Academia-0026</t>
+          <t>Poster-Academia-0081</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -8536,10 +8548,14 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>406909164941</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr"/>
+          <t>406902627420</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="L153" t="inlineStr">
         <is>
           <t>True</t>
@@ -8548,167 +8564,163 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Poster-Academia-0027</t>
+          <t>Acrylic-Grimdark-0012</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>No safe action under current weak-network protocol.</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>406909216787</t>
+          <t>406909148324</t>
         </is>
       </c>
       <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Poster-Academia-0028</t>
+          <t>Acrylic-Grimdark-0013</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>No safe action under current weak-network protocol.</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I155" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>406909220927</t>
+          <t>406909151733</t>
         </is>
       </c>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Poster-Academia-0081</t>
+          <t>Acrylic-Grimdark-0015</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Etsy_Draft_Prepared</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>KEEP_FOR_ETSY_PHASE1</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Candidate already selected for Etsy relaunch; wait for shop/OAuth readiness and listing-fee confirmation.</t>
+          <t>No safe action under current weak-network protocol.</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>local</t>
         </is>
       </c>
       <c r="I156" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>406902627420</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>406909166683</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8730,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0012</t>
+          <t>Acrylic-Grimdark-0017</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -8756,7 +8768,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>406909148324</t>
+          <t>406909219066</t>
         </is>
       </c>
       <c r="K157" t="inlineStr"/>
@@ -8772,7 +8784,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0013</t>
+          <t>Acrylic-Grimdark-0018</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -8810,7 +8822,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>406909151733</t>
+          <t>406909222169</t>
         </is>
       </c>
       <c r="K158" t="inlineStr"/>
@@ -8826,7 +8838,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0015</t>
+          <t>Acrylic-Grimdark-0021</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8864,7 +8876,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>406909166683</t>
+          <t>406909225478</t>
         </is>
       </c>
       <c r="K159" t="inlineStr"/>
@@ -8880,7 +8892,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0017</t>
+          <t>Acrylic-Grimdark-0022</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8918,7 +8930,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>406909219066</t>
+          <t>406909226531</t>
         </is>
       </c>
       <c r="K160" t="inlineStr"/>
@@ -8934,7 +8946,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0018</t>
+          <t>Acrylic-Grimdark-0023</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -8972,7 +8984,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>406909222169</t>
+          <t>406909228840</t>
         </is>
       </c>
       <c r="K161" t="inlineStr"/>
@@ -8988,7 +9000,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0021</t>
+          <t>Acrylic-Grimdark-0024</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -9026,7 +9038,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>406909225478</t>
+          <t>406909231370</t>
         </is>
       </c>
       <c r="K162" t="inlineStr"/>
@@ -9042,7 +9054,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0022</t>
+          <t>Acrylic-Grimdark-0025</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -9080,7 +9092,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>406909226531</t>
+          <t>406909232068</t>
         </is>
       </c>
       <c r="K163" t="inlineStr"/>
@@ -9096,7 +9108,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0023</t>
+          <t>Acrylic-Grimdark-0026</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -9134,7 +9146,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>406909228840</t>
+          <t>406909232951</t>
         </is>
       </c>
       <c r="K164" t="inlineStr"/>
@@ -9150,7 +9162,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0024</t>
+          <t>Acrylic-Grimdark-0028</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -9188,7 +9200,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>406909231370</t>
+          <t>406909234435</t>
         </is>
       </c>
       <c r="K165" t="inlineStr"/>
@@ -9204,7 +9216,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0025</t>
+          <t>Acrylic-Grimdark-0032</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -9242,7 +9254,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>406909232068</t>
+          <t>406909238227</t>
         </is>
       </c>
       <c r="K166" t="inlineStr"/>
@@ -9258,7 +9270,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0026</t>
+          <t>Acrylic-Grimdark-0034</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -9296,7 +9308,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>406909232951</t>
+          <t>406909242546</t>
         </is>
       </c>
       <c r="K167" t="inlineStr"/>
@@ -9312,7 +9324,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0028</t>
+          <t>Acrylic-Grimdark-0036</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -9350,7 +9362,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>406909234435</t>
+          <t>406909244688</t>
         </is>
       </c>
       <c r="K168" t="inlineStr"/>
@@ -9366,7 +9378,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0032</t>
+          <t>Acrylic-Grimdark-0037</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -9404,7 +9416,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>406909238227</t>
+          <t>406909247161</t>
         </is>
       </c>
       <c r="K169" t="inlineStr"/>
@@ -9420,7 +9432,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0034</t>
+          <t>Acrylic-Zen-0004</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -9430,7 +9442,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -9458,10 +9470,14 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>406909242546</t>
-        </is>
-      </c>
-      <c r="K170" t="inlineStr"/>
+          <t>406902888077</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L170" t="inlineStr">
         <is>
           <t>False</t>
@@ -9474,17 +9490,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0036</t>
+          <t>Poster-Academia-0001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -9512,10 +9528,14 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>406909244688</t>
-        </is>
-      </c>
-      <c r="K171" t="inlineStr"/>
+          <t>406902584620</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L171" t="inlineStr">
         <is>
           <t>False</t>
@@ -9528,17 +9548,17 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Acrylic-Grimdark-0037</t>
+          <t>Poster-Academia-0001-FIX1</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -9566,7 +9586,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>406909247161</t>
+          <t>406911589289</t>
         </is>
       </c>
       <c r="K172" t="inlineStr"/>
@@ -9582,17 +9602,17 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Acrylic-Zen-0004</t>
+          <t>Poster-Academia-0023</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -9620,14 +9640,10 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>406902888077</t>
-        </is>
-      </c>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>406909147173</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr">
         <is>
           <t>False</t>
@@ -9640,7 +9656,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Poster-Academia-0001</t>
+          <t>Poster-Academia-0024</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -9678,14 +9694,10 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>406902584620</t>
-        </is>
-      </c>
-      <c r="K174" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>406909150037</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr"/>
       <c r="L174" t="inlineStr">
         <is>
           <t>False</t>
@@ -9698,7 +9710,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Poster-Academia-0001-FIX1</t>
+          <t>Poster-Academia-0025</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -9736,7 +9748,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>406911589289</t>
+          <t>406909153504</t>
         </is>
       </c>
       <c r="K175" t="inlineStr"/>
@@ -9752,7 +9764,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Poster-Academia-0023</t>
+          <t>Poster-Academia-0030</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -9790,7 +9802,7 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>406909147173</t>
+          <t>406909264998</t>
         </is>
       </c>
       <c r="K176" t="inlineStr"/>
@@ -9806,7 +9818,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Poster-Academia-0024</t>
+          <t>Poster-Academia-0031</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -9844,7 +9856,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>406909150037</t>
+          <t>406909266188</t>
         </is>
       </c>
       <c r="K177" t="inlineStr"/>
@@ -9860,7 +9872,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Poster-Academia-0025</t>
+          <t>Poster-Academia-0032</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -9898,7 +9910,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>406909153504</t>
+          <t>406909268494</t>
         </is>
       </c>
       <c r="K178" t="inlineStr"/>
@@ -9914,7 +9926,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Poster-Academia-0030</t>
+          <t>Poster-Academia-0033</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -9952,7 +9964,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>406909264998</t>
+          <t>406909269321</t>
         </is>
       </c>
       <c r="K179" t="inlineStr"/>
@@ -9968,7 +9980,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Poster-Academia-0031</t>
+          <t>Poster-Academia-0034</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -10006,7 +10018,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>406909266188</t>
+          <t>406909467980</t>
         </is>
       </c>
       <c r="K180" t="inlineStr"/>
@@ -10022,7 +10034,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Poster-Academia-0032</t>
+          <t>Poster-Academia-0035</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -10060,7 +10072,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>406909268494</t>
+          <t>406909471020</t>
         </is>
       </c>
       <c r="K181" t="inlineStr"/>
@@ -10076,7 +10088,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Poster-Academia-0033</t>
+          <t>Poster-Academia-0037</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -10114,7 +10126,7 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>406909269321</t>
+          <t>406909473606</t>
         </is>
       </c>
       <c r="K182" t="inlineStr"/>
@@ -10130,7 +10142,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Poster-Academia-0034</t>
+          <t>Poster-Academia-0038</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -10168,7 +10180,7 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>406909467980</t>
+          <t>406910056059</t>
         </is>
       </c>
       <c r="K183" t="inlineStr"/>
@@ -10184,7 +10196,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Poster-Academia-0035</t>
+          <t>Poster-Academia-0039</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -10222,7 +10234,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>406909471020</t>
+          <t>406910057355</t>
         </is>
       </c>
       <c r="K184" t="inlineStr"/>
@@ -10238,7 +10250,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Poster-Academia-0037</t>
+          <t>Poster-Academia-0040</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -10276,7 +10288,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>406909473606</t>
+          <t>406910058626</t>
         </is>
       </c>
       <c r="K185" t="inlineStr"/>
@@ -10292,7 +10304,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Poster-Academia-0038</t>
+          <t>Poster-Academia-0041</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -10330,7 +10342,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>406910056059</t>
+          <t>406910059060</t>
         </is>
       </c>
       <c r="K186" t="inlineStr"/>
@@ -10346,7 +10358,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Poster-Academia-0039</t>
+          <t>Poster-Academia-0042</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -10384,7 +10396,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>406910057355</t>
+          <t>406910060084</t>
         </is>
       </c>
       <c r="K187" t="inlineStr"/>
@@ -10400,7 +10412,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Poster-Academia-0040</t>
+          <t>Poster-Academia-0082</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -10438,10 +10450,14 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>406910058626</t>
-        </is>
-      </c>
-      <c r="K188" t="inlineStr"/>
+          <t>406902648209</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="L188" t="inlineStr">
         <is>
           <t>False</t>
@@ -10454,7 +10470,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Poster-Academia-0041</t>
+          <t>Poster-Academia-0085</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -10492,10 +10508,14 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>406910059060</t>
-        </is>
-      </c>
-      <c r="K189" t="inlineStr"/>
+          <t>406902882943</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="L189" t="inlineStr">
         <is>
           <t>False</t>
@@ -10508,7 +10528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Poster-Academia-0042</t>
+          <t>Poster-Zen-0003</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -10518,7 +10538,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -10544,11 +10564,7 @@
       <c r="I190" t="b">
         <v>1</v>
       </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t>406910060084</t>
-        </is>
-      </c>
+      <c r="J190" t="inlineStr"/>
       <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr">
         <is>
@@ -10562,12 +10578,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Poster-Academia-0082</t>
+          <t>Sticker-Academia-0004</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -10600,12 +10616,12 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>406902648209</t>
+          <t>406892408950</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L191" t="inlineStr">
@@ -10620,12 +10636,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Poster-Academia-0085</t>
+          <t>Sticker-Academia-0005</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -10656,16 +10672,8 @@
       <c r="I192" t="b">
         <v>1</v>
       </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t>406902882943</t>
-        </is>
-      </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr">
         <is>
           <t>False</t>
@@ -10678,17 +10686,17 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Poster-Zen-0003</t>
+          <t>Sticker-Academia-0005-FIX1</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Zen</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -10728,7 +10736,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0004</t>
+          <t>Sticker-Academia-0006</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -10764,16 +10772,8 @@
       <c r="I194" t="b">
         <v>1</v>
       </c>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t>406892408950</t>
-        </is>
-      </c>
-      <c r="K194" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
       <c r="L194" t="inlineStr">
         <is>
           <t>False</t>
@@ -10786,7 +10786,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0005</t>
+          <t>Sticker-Academia-0006-FIX1</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -10822,7 +10822,11 @@
       <c r="I195" t="b">
         <v>1</v>
       </c>
-      <c r="J195" t="inlineStr"/>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>406909095974</t>
+        </is>
+      </c>
       <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr">
         <is>
@@ -10836,7 +10840,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0005-FIX1</t>
+          <t>Sticker-Academia-0007</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -10886,7 +10890,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0006</t>
+          <t>Sticker-Academia-0007-FIX1</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -10922,7 +10926,11 @@
       <c r="I197" t="b">
         <v>1</v>
       </c>
-      <c r="J197" t="inlineStr"/>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>406909097469</t>
+        </is>
+      </c>
       <c r="K197" t="inlineStr"/>
       <c r="L197" t="inlineStr">
         <is>
@@ -10936,7 +10944,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0006-FIX1</t>
+          <t>Sticker-Academia-0008</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -10972,11 +10980,7 @@
       <c r="I198" t="b">
         <v>1</v>
       </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t>406909095974</t>
-        </is>
-      </c>
+      <c r="J198" t="inlineStr"/>
       <c r="K198" t="inlineStr"/>
       <c r="L198" t="inlineStr">
         <is>
@@ -10990,7 +10994,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0007</t>
+          <t>Sticker-Academia-0008-FIX1</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -11026,7 +11030,11 @@
       <c r="I199" t="b">
         <v>1</v>
       </c>
-      <c r="J199" t="inlineStr"/>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>406909100892</t>
+        </is>
+      </c>
       <c r="K199" t="inlineStr"/>
       <c r="L199" t="inlineStr">
         <is>
@@ -11040,7 +11048,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0007-FIX1</t>
+          <t>Sticker-Academia-0009</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -11076,11 +11084,7 @@
       <c r="I200" t="b">
         <v>1</v>
       </c>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t>406909097469</t>
-        </is>
-      </c>
+      <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr"/>
       <c r="L200" t="inlineStr">
         <is>
@@ -11094,7 +11098,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0008</t>
+          <t>Sticker-Academia-0009-FIX1</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -11130,7 +11134,11 @@
       <c r="I201" t="b">
         <v>1</v>
       </c>
-      <c r="J201" t="inlineStr"/>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>406909114799</t>
+        </is>
+      </c>
       <c r="K201" t="inlineStr"/>
       <c r="L201" t="inlineStr">
         <is>
@@ -11144,7 +11152,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0008-FIX1</t>
+          <t>Sticker-Academia-0010</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -11180,11 +11188,7 @@
       <c r="I202" t="b">
         <v>1</v>
       </c>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t>406909100892</t>
-        </is>
-      </c>
+      <c r="J202" t="inlineStr"/>
       <c r="K202" t="inlineStr"/>
       <c r="L202" t="inlineStr">
         <is>
@@ -11198,7 +11202,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0009</t>
+          <t>Sticker-Academia-0010-FIX1</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -11234,7 +11238,11 @@
       <c r="I203" t="b">
         <v>1</v>
       </c>
-      <c r="J203" t="inlineStr"/>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>406909116716</t>
+        </is>
+      </c>
       <c r="K203" t="inlineStr"/>
       <c r="L203" t="inlineStr">
         <is>
@@ -11248,7 +11256,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0009-FIX1</t>
+          <t>Sticker-Academia-0011</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -11284,11 +11292,7 @@
       <c r="I204" t="b">
         <v>1</v>
       </c>
-      <c r="J204" t="inlineStr">
-        <is>
-          <t>406909114799</t>
-        </is>
-      </c>
+      <c r="J204" t="inlineStr"/>
       <c r="K204" t="inlineStr"/>
       <c r="L204" t="inlineStr">
         <is>
@@ -11302,7 +11306,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0010</t>
+          <t>Sticker-Academia-0011-FIX1</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -11338,7 +11342,11 @@
       <c r="I205" t="b">
         <v>1</v>
       </c>
-      <c r="J205" t="inlineStr"/>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>406909118000</t>
+        </is>
+      </c>
       <c r="K205" t="inlineStr"/>
       <c r="L205" t="inlineStr">
         <is>
@@ -11352,7 +11360,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0010-FIX1</t>
+          <t>Sticker-Academia-0014</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -11388,11 +11396,7 @@
       <c r="I206" t="b">
         <v>1</v>
       </c>
-      <c r="J206" t="inlineStr">
-        <is>
-          <t>406909116716</t>
-        </is>
-      </c>
+      <c r="J206" t="inlineStr"/>
       <c r="K206" t="inlineStr"/>
       <c r="L206" t="inlineStr">
         <is>
@@ -11406,7 +11410,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0011</t>
+          <t>Sticker-Academia-0014-FIX1</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -11442,7 +11446,11 @@
       <c r="I207" t="b">
         <v>1</v>
       </c>
-      <c r="J207" t="inlineStr"/>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>406909119544</t>
+        </is>
+      </c>
       <c r="K207" t="inlineStr"/>
       <c r="L207" t="inlineStr">
         <is>
@@ -11456,7 +11464,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0011-FIX1</t>
+          <t>Sticker-Academia-0015</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -11492,11 +11500,7 @@
       <c r="I208" t="b">
         <v>1</v>
       </c>
-      <c r="J208" t="inlineStr">
-        <is>
-          <t>406909118000</t>
-        </is>
-      </c>
+      <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr"/>
       <c r="L208" t="inlineStr">
         <is>
@@ -11510,7 +11514,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0014</t>
+          <t>Sticker-Academia-0015-FIX1</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -11546,7 +11550,11 @@
       <c r="I209" t="b">
         <v>1</v>
       </c>
-      <c r="J209" t="inlineStr"/>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>406909121336</t>
+        </is>
+      </c>
       <c r="K209" t="inlineStr"/>
       <c r="L209" t="inlineStr">
         <is>
@@ -11560,7 +11568,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0014-FIX1</t>
+          <t>Sticker-Academia-0016</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -11596,11 +11604,7 @@
       <c r="I210" t="b">
         <v>1</v>
       </c>
-      <c r="J210" t="inlineStr">
-        <is>
-          <t>406909119544</t>
-        </is>
-      </c>
+      <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr"/>
       <c r="L210" t="inlineStr">
         <is>
@@ -11614,7 +11618,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0015</t>
+          <t>Sticker-Academia-0016-FIX1</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -11650,7 +11654,11 @@
       <c r="I211" t="b">
         <v>1</v>
       </c>
-      <c r="J211" t="inlineStr"/>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>406909122790</t>
+        </is>
+      </c>
       <c r="K211" t="inlineStr"/>
       <c r="L211" t="inlineStr">
         <is>
@@ -11664,7 +11672,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0015-FIX1</t>
+          <t>Sticker-Zen-0001</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -11674,7 +11682,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -11700,11 +11708,7 @@
       <c r="I212" t="b">
         <v>1</v>
       </c>
-      <c r="J212" t="inlineStr">
-        <is>
-          <t>406909121336</t>
-        </is>
-      </c>
+      <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr"/>
       <c r="L212" t="inlineStr">
         <is>
@@ -11718,7 +11722,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0016</t>
+          <t>Sticker-Zen-0001-FIX1</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -11728,7 +11732,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -11754,7 +11758,11 @@
       <c r="I213" t="b">
         <v>1</v>
       </c>
-      <c r="J213" t="inlineStr"/>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>406909124585</t>
+        </is>
+      </c>
       <c r="K213" t="inlineStr"/>
       <c r="L213" t="inlineStr">
         <is>
@@ -11768,7 +11776,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Sticker-Academia-0016-FIX1</t>
+          <t>Sticker-Zen-0002</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -11778,7 +11786,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Zen</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -11804,11 +11812,7 @@
       <c r="I214" t="b">
         <v>1</v>
       </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>406909122790</t>
-        </is>
-      </c>
+      <c r="J214" t="inlineStr"/>
       <c r="K214" t="inlineStr"/>
       <c r="L214" t="inlineStr">
         <is>
@@ -11822,7 +11826,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0001</t>
+          <t>Sticker-Zen-0002-FIX1</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -11858,7 +11862,11 @@
       <c r="I215" t="b">
         <v>1</v>
       </c>
-      <c r="J215" t="inlineStr"/>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>406909125700</t>
+        </is>
+      </c>
       <c r="K215" t="inlineStr"/>
       <c r="L215" t="inlineStr">
         <is>
@@ -11872,7 +11880,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0001-FIX1</t>
+          <t>Sticker-Zen-0003</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -11908,11 +11916,7 @@
       <c r="I216" t="b">
         <v>1</v>
       </c>
-      <c r="J216" t="inlineStr">
-        <is>
-          <t>406909124585</t>
-        </is>
-      </c>
+      <c r="J216" t="inlineStr"/>
       <c r="K216" t="inlineStr"/>
       <c r="L216" t="inlineStr">
         <is>
@@ -11926,7 +11930,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0002</t>
+          <t>Sticker-Zen-0003-FIX1</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -11962,7 +11966,11 @@
       <c r="I217" t="b">
         <v>1</v>
       </c>
-      <c r="J217" t="inlineStr"/>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>406909126789</t>
+        </is>
+      </c>
       <c r="K217" t="inlineStr"/>
       <c r="L217" t="inlineStr">
         <is>
@@ -11976,7 +11984,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0002-FIX1</t>
+          <t>Sticker-Zen-0004</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -12012,11 +12020,7 @@
       <c r="I218" t="b">
         <v>1</v>
       </c>
-      <c r="J218" t="inlineStr">
-        <is>
-          <t>406909125700</t>
-        </is>
-      </c>
+      <c r="J218" t="inlineStr"/>
       <c r="K218" t="inlineStr"/>
       <c r="L218" t="inlineStr">
         <is>
@@ -12030,7 +12034,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0003</t>
+          <t>Sticker-Zen-0004-FIX1</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -12066,7 +12070,11 @@
       <c r="I219" t="b">
         <v>1</v>
       </c>
-      <c r="J219" t="inlineStr"/>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>406909127704</t>
+        </is>
+      </c>
       <c r="K219" t="inlineStr"/>
       <c r="L219" t="inlineStr">
         <is>
@@ -12080,7 +12088,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0003-FIX1</t>
+          <t>Sticker-Zen-0005</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -12116,11 +12124,7 @@
       <c r="I220" t="b">
         <v>1</v>
       </c>
-      <c r="J220" t="inlineStr">
-        <is>
-          <t>406909126789</t>
-        </is>
-      </c>
+      <c r="J220" t="inlineStr"/>
       <c r="K220" t="inlineStr"/>
       <c r="L220" t="inlineStr">
         <is>
@@ -12134,7 +12138,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0004</t>
+          <t>Sticker-Zen-0005-FIX1</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -12170,7 +12174,11 @@
       <c r="I221" t="b">
         <v>1</v>
       </c>
-      <c r="J221" t="inlineStr"/>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>406909342825</t>
+        </is>
+      </c>
       <c r="K221" t="inlineStr"/>
       <c r="L221" t="inlineStr">
         <is>
@@ -12184,7 +12192,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0004-FIX1</t>
+          <t>Sticker-Zen-0007</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -12220,11 +12228,7 @@
       <c r="I222" t="b">
         <v>1</v>
       </c>
-      <c r="J222" t="inlineStr">
-        <is>
-          <t>406909127704</t>
-        </is>
-      </c>
+      <c r="J222" t="inlineStr"/>
       <c r="K222" t="inlineStr"/>
       <c r="L222" t="inlineStr">
         <is>
@@ -12238,7 +12242,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0005</t>
+          <t>Sticker-Zen-0007-FIX1</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -12274,7 +12278,11 @@
       <c r="I223" t="b">
         <v>1</v>
       </c>
-      <c r="J223" t="inlineStr"/>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>406909344491</t>
+        </is>
+      </c>
       <c r="K223" t="inlineStr"/>
       <c r="L223" t="inlineStr">
         <is>
@@ -12288,7 +12296,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0005-FIX1</t>
+          <t>Sticker-Zen-0008</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -12324,11 +12332,7 @@
       <c r="I224" t="b">
         <v>1</v>
       </c>
-      <c r="J224" t="inlineStr">
-        <is>
-          <t>406909342825</t>
-        </is>
-      </c>
+      <c r="J224" t="inlineStr"/>
       <c r="K224" t="inlineStr"/>
       <c r="L224" t="inlineStr">
         <is>
@@ -12342,7 +12346,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0007</t>
+          <t>Sticker-Zen-0008-FIX1</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -12378,7 +12382,11 @@
       <c r="I225" t="b">
         <v>1</v>
       </c>
-      <c r="J225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>406909345291</t>
+        </is>
+      </c>
       <c r="K225" t="inlineStr"/>
       <c r="L225" t="inlineStr">
         <is>
@@ -12392,7 +12400,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0007-FIX1</t>
+          <t>Sticker-Zen-0009</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -12428,11 +12436,7 @@
       <c r="I226" t="b">
         <v>1</v>
       </c>
-      <c r="J226" t="inlineStr">
-        <is>
-          <t>406909344491</t>
-        </is>
-      </c>
+      <c r="J226" t="inlineStr"/>
       <c r="K226" t="inlineStr"/>
       <c r="L226" t="inlineStr">
         <is>
@@ -12446,7 +12450,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0008</t>
+          <t>Sticker-Zen-0009-FIX1</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -12482,7 +12486,11 @@
       <c r="I227" t="b">
         <v>1</v>
       </c>
-      <c r="J227" t="inlineStr"/>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>406909353931</t>
+        </is>
+      </c>
       <c r="K227" t="inlineStr"/>
       <c r="L227" t="inlineStr">
         <is>
@@ -12496,7 +12504,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0008-FIX1</t>
+          <t>Sticker-Zen-0022</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -12532,11 +12540,7 @@
       <c r="I228" t="b">
         <v>1</v>
       </c>
-      <c r="J228" t="inlineStr">
-        <is>
-          <t>406909345291</t>
-        </is>
-      </c>
+      <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr"/>
       <c r="L228" t="inlineStr">
         <is>
@@ -12550,7 +12554,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0009</t>
+          <t>Sticker-Zen-0022-FIX1</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -12586,7 +12590,11 @@
       <c r="I229" t="b">
         <v>1</v>
       </c>
-      <c r="J229" t="inlineStr"/>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>406909354903</t>
+        </is>
+      </c>
       <c r="K229" t="inlineStr"/>
       <c r="L229" t="inlineStr">
         <is>
@@ -12600,7 +12608,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0009-FIX1</t>
+          <t>Sticker-Zen-0024</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -12636,11 +12644,7 @@
       <c r="I230" t="b">
         <v>1</v>
       </c>
-      <c r="J230" t="inlineStr">
-        <is>
-          <t>406909353931</t>
-        </is>
-      </c>
+      <c r="J230" t="inlineStr"/>
       <c r="K230" t="inlineStr"/>
       <c r="L230" t="inlineStr">
         <is>
@@ -12654,7 +12658,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0022</t>
+          <t>Sticker-Zen-0024-FIX1</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -12690,7 +12694,11 @@
       <c r="I231" t="b">
         <v>1</v>
       </c>
-      <c r="J231" t="inlineStr"/>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>406909355853</t>
+        </is>
+      </c>
       <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr">
         <is>
@@ -12704,7 +12712,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0022-FIX1</t>
+          <t>Sticker-Zen-0025</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -12740,11 +12748,7 @@
       <c r="I232" t="b">
         <v>1</v>
       </c>
-      <c r="J232" t="inlineStr">
-        <is>
-          <t>406909354903</t>
-        </is>
-      </c>
+      <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr"/>
       <c r="L232" t="inlineStr">
         <is>
@@ -12758,7 +12762,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0024</t>
+          <t>Sticker-Zen-0025-FIX1</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -12794,7 +12798,11 @@
       <c r="I233" t="b">
         <v>1</v>
       </c>
-      <c r="J233" t="inlineStr"/>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>406909359949</t>
+        </is>
+      </c>
       <c r="K233" t="inlineStr"/>
       <c r="L233" t="inlineStr">
         <is>
@@ -12808,7 +12816,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0024-FIX1</t>
+          <t>Sticker-Zen-0026</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -12844,11 +12852,7 @@
       <c r="I234" t="b">
         <v>1</v>
       </c>
-      <c r="J234" t="inlineStr">
-        <is>
-          <t>406909355853</t>
-        </is>
-      </c>
+      <c r="J234" t="inlineStr"/>
       <c r="K234" t="inlineStr"/>
       <c r="L234" t="inlineStr">
         <is>
@@ -12862,7 +12866,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0025</t>
+          <t>Sticker-Zen-0027</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -12912,7 +12916,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0025-FIX1</t>
+          <t>Sticker-Zen-0027-FIX1</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -12950,7 +12954,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>406909359949</t>
+          <t>406909364977</t>
         </is>
       </c>
       <c r="K236" t="inlineStr"/>
@@ -12966,7 +12970,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0026</t>
+          <t>Sticker-Zen-0029</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -13016,7 +13020,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0027</t>
+          <t>Sticker-Zen-0031</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -13066,7 +13070,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0027-FIX1</t>
+          <t>Sticker-Zen-0032</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -13102,11 +13106,7 @@
       <c r="I239" t="b">
         <v>1</v>
       </c>
-      <c r="J239" t="inlineStr">
-        <is>
-          <t>406909364977</t>
-        </is>
-      </c>
+      <c r="J239" t="inlineStr"/>
       <c r="K239" t="inlineStr"/>
       <c r="L239" t="inlineStr">
         <is>
@@ -13120,7 +13120,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0029</t>
+          <t>Sticker-Zen-0034</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0031</t>
+          <t>Sticker-Zen-0035</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -13220,7 +13220,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0032</t>
+          <t>Sticker-Zen-0036</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0034</t>
+          <t>Sticker-Zen-0037</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0035</t>
+          <t>Sticker-Zen-0038</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -13370,7 +13370,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0036</t>
+          <t>Sticker-Zen-0040</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -13420,7 +13420,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0037</t>
+          <t>Sticker-Zen-0041</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -13470,7 +13470,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0038</t>
+          <t>Sticker-Zen-0041-FIX1</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -13506,7 +13506,11 @@
       <c r="I247" t="b">
         <v>1</v>
       </c>
-      <c r="J247" t="inlineStr"/>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>406909368739</t>
+        </is>
+      </c>
       <c r="K247" t="inlineStr"/>
       <c r="L247" t="inlineStr">
         <is>
@@ -13520,7 +13524,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0040</t>
+          <t>Sticker-Zen-0042</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -13570,7 +13574,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0041</t>
+          <t>Sticker-Zen-0042-FIX1</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -13606,7 +13610,11 @@
       <c r="I249" t="b">
         <v>1</v>
       </c>
-      <c r="J249" t="inlineStr"/>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>406909373586</t>
+        </is>
+      </c>
       <c r="K249" t="inlineStr"/>
       <c r="L249" t="inlineStr">
         <is>
@@ -13620,7 +13628,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0041-FIX1</t>
+          <t>Sticker-Zen-0044</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -13658,10 +13666,14 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>406909368739</t>
-        </is>
-      </c>
-      <c r="K250" t="inlineStr"/>
+          <t>406902622710</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L250" t="inlineStr">
         <is>
           <t>False</t>
@@ -13674,7 +13686,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0042</t>
+          <t>Sticker-Zen-0044-FIX1</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -13710,7 +13722,11 @@
       <c r="I251" t="b">
         <v>1</v>
       </c>
-      <c r="J251" t="inlineStr"/>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>406909884756</t>
+        </is>
+      </c>
       <c r="K251" t="inlineStr"/>
       <c r="L251" t="inlineStr">
         <is>
@@ -13724,7 +13740,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0042-FIX1</t>
+          <t>Sticker-Zen-0045</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -13762,10 +13778,14 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>406909373586</t>
-        </is>
-      </c>
-      <c r="K252" t="inlineStr"/>
+          <t>406902640998</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L252" t="inlineStr">
         <is>
           <t>False</t>
@@ -13778,7 +13798,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0044</t>
+          <t>Sticker-Zen-0045-FIX1</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -13816,14 +13836,10 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>406902622710</t>
-        </is>
-      </c>
-      <c r="K253" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909890800</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr"/>
       <c r="L253" t="inlineStr">
         <is>
           <t>False</t>
@@ -13836,7 +13852,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0044-FIX1</t>
+          <t>Sticker-Zen-0046</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -13874,10 +13890,14 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>406909884756</t>
-        </is>
-      </c>
-      <c r="K254" t="inlineStr"/>
+          <t>406902663232</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L254" t="inlineStr">
         <is>
           <t>False</t>
@@ -13890,7 +13910,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0045</t>
+          <t>Sticker-Zen-0046-FIX1</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -13928,14 +13948,10 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>406902640998</t>
-        </is>
-      </c>
-      <c r="K255" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909891985</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr"/>
       <c r="L255" t="inlineStr">
         <is>
           <t>False</t>
@@ -13948,7 +13964,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0045-FIX1</t>
+          <t>Sticker-Zen-0048</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -13984,11 +14000,7 @@
       <c r="I256" t="b">
         <v>1</v>
       </c>
-      <c r="J256" t="inlineStr">
-        <is>
-          <t>406909890800</t>
-        </is>
-      </c>
+      <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr"/>
       <c r="L256" t="inlineStr">
         <is>
@@ -14002,7 +14014,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0046</t>
+          <t>Sticker-Zen-0049</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -14040,7 +14052,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>406902663232</t>
+          <t>406902713267</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -14060,7 +14072,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0046-FIX1</t>
+          <t>Sticker-Zen-0049-FIX1</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -14098,7 +14110,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>406909891985</t>
+          <t>406909893702</t>
         </is>
       </c>
       <c r="K258" t="inlineStr"/>
@@ -14114,7 +14126,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0048</t>
+          <t>Sticker-Zen-0050</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -14150,8 +14162,16 @@
       <c r="I259" t="b">
         <v>1</v>
       </c>
-      <c r="J259" t="inlineStr"/>
-      <c r="K259" t="inlineStr"/>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>406902886081</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L259" t="inlineStr">
         <is>
           <t>False</t>
@@ -14164,7 +14184,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0049</t>
+          <t>Sticker-Zen-0050-FIX1</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -14202,14 +14222,10 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>406902713267</t>
-        </is>
-      </c>
-      <c r="K260" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909904704</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr"/>
       <c r="L260" t="inlineStr">
         <is>
           <t>False</t>
@@ -14222,7 +14238,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0049-FIX1</t>
+          <t>Sticker-Zen-0051</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -14260,10 +14276,14 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>406909893702</t>
-        </is>
-      </c>
-      <c r="K261" t="inlineStr"/>
+          <t>406902889638</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L261" t="inlineStr">
         <is>
           <t>False</t>
@@ -14276,7 +14296,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0050</t>
+          <t>Sticker-Zen-0051-FIX1</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -14314,14 +14334,10 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>406902886081</t>
-        </is>
-      </c>
-      <c r="K262" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909905683</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr"/>
       <c r="L262" t="inlineStr">
         <is>
           <t>False</t>
@@ -14334,7 +14350,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0050-FIX1</t>
+          <t>Sticker-Zen-0052</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -14372,10 +14388,14 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>406909904704</t>
-        </is>
-      </c>
-      <c r="K263" t="inlineStr"/>
+          <t>406902896387</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L263" t="inlineStr">
         <is>
           <t>False</t>
@@ -14388,7 +14408,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0051</t>
+          <t>Sticker-Zen-0052-FIX1</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -14426,14 +14446,10 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>406902889638</t>
-        </is>
-      </c>
-      <c r="K264" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909906686</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr"/>
       <c r="L264" t="inlineStr">
         <is>
           <t>False</t>
@@ -14446,7 +14462,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0051-FIX1</t>
+          <t>Sticker-Zen-0053</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -14484,10 +14500,14 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>406909905683</t>
-        </is>
-      </c>
-      <c r="K265" t="inlineStr"/>
+          <t>406902900109</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L265" t="inlineStr">
         <is>
           <t>False</t>
@@ -14500,7 +14520,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0052</t>
+          <t>Sticker-Zen-0053-FIX1</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -14538,14 +14558,10 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>406902896387</t>
-        </is>
-      </c>
-      <c r="K266" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909907111</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr"/>
       <c r="L266" t="inlineStr">
         <is>
           <t>False</t>
@@ -14558,7 +14574,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0052-FIX1</t>
+          <t>Sticker-Zen-0054</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -14596,10 +14612,14 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>406909906686</t>
-        </is>
-      </c>
-      <c r="K267" t="inlineStr"/>
+          <t>406903032635</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L267" t="inlineStr">
         <is>
           <t>False</t>
@@ -14612,7 +14632,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0053</t>
+          <t>Sticker-Zen-0054-FIX1</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -14650,14 +14670,10 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>406902900109</t>
-        </is>
-      </c>
-      <c r="K268" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406909907742</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr"/>
       <c r="L268" t="inlineStr">
         <is>
           <t>False</t>
@@ -14670,7 +14686,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0053-FIX1</t>
+          <t>Sticker-Zen-0055</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -14708,10 +14724,14 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>406909907111</t>
-        </is>
-      </c>
-      <c r="K269" t="inlineStr"/>
+          <t>406903037933</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L269" t="inlineStr">
         <is>
           <t>False</t>
@@ -14724,7 +14744,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0054</t>
+          <t>Sticker-Zen-0055-FIX1</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -14762,14 +14782,10 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>406903032635</t>
-        </is>
-      </c>
-      <c r="K270" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406910984204</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr"/>
       <c r="L270" t="inlineStr">
         <is>
           <t>False</t>
@@ -14782,7 +14798,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0054-FIX1</t>
+          <t>Sticker-Zen-0056</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -14820,10 +14836,14 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>406909907742</t>
-        </is>
-      </c>
-      <c r="K271" t="inlineStr"/>
+          <t>406903041315</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L271" t="inlineStr">
         <is>
           <t>False</t>
@@ -14836,7 +14856,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0055</t>
+          <t>Sticker-Zen-0056-FIX1</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -14874,14 +14894,10 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>406903037933</t>
-        </is>
-      </c>
-      <c r="K272" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911030956</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr"/>
       <c r="L272" t="inlineStr">
         <is>
           <t>False</t>
@@ -14894,7 +14910,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0055-FIX1</t>
+          <t>Sticker-Zen-0057</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -14932,10 +14948,14 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>406910984204</t>
-        </is>
-      </c>
-      <c r="K273" t="inlineStr"/>
+          <t>406903044643</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L273" t="inlineStr">
         <is>
           <t>False</t>
@@ -14948,7 +14968,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0056</t>
+          <t>Sticker-Zen-0057-FIX1</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -14986,14 +15006,10 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>406903041315</t>
-        </is>
-      </c>
-      <c r="K274" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911046712</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr"/>
       <c r="L274" t="inlineStr">
         <is>
           <t>False</t>
@@ -15006,7 +15022,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0056-FIX1</t>
+          <t>Sticker-Zen-0058</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -15044,10 +15060,14 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>406911030956</t>
-        </is>
-      </c>
-      <c r="K275" t="inlineStr"/>
+          <t>406903049411</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L275" t="inlineStr">
         <is>
           <t>False</t>
@@ -15060,7 +15080,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0057</t>
+          <t>Sticker-Zen-0058-FIX1</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -15098,14 +15118,10 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>406903044643</t>
-        </is>
-      </c>
-      <c r="K276" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911102240</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr"/>
       <c r="L276" t="inlineStr">
         <is>
           <t>False</t>
@@ -15118,7 +15134,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0057-FIX1</t>
+          <t>Sticker-Zen-0060</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -15156,10 +15172,14 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>406911046712</t>
-        </is>
-      </c>
-      <c r="K277" t="inlineStr"/>
+          <t>406903249053</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L277" t="inlineStr">
         <is>
           <t>False</t>
@@ -15172,7 +15192,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0058</t>
+          <t>Sticker-Zen-0060-FIX1</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -15210,14 +15230,10 @@
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>406903049411</t>
-        </is>
-      </c>
-      <c r="K278" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911120974</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr"/>
       <c r="L278" t="inlineStr">
         <is>
           <t>False</t>
@@ -15230,7 +15246,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0058-FIX1</t>
+          <t>Sticker-Zen-0061</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -15268,10 +15284,14 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>406911102240</t>
-        </is>
-      </c>
-      <c r="K279" t="inlineStr"/>
+          <t>406903249987</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L279" t="inlineStr">
         <is>
           <t>False</t>
@@ -15284,7 +15304,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0060</t>
+          <t>Sticker-Zen-0061-FIX1</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -15322,14 +15342,10 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>406903249053</t>
-        </is>
-      </c>
-      <c r="K280" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911452547</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr"/>
       <c r="L280" t="inlineStr">
         <is>
           <t>False</t>
@@ -15342,7 +15358,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0060-FIX1</t>
+          <t>Sticker-Zen-0062</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -15380,10 +15396,14 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>406911120974</t>
-        </is>
-      </c>
-      <c r="K281" t="inlineStr"/>
+          <t>406903250891</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L281" t="inlineStr">
         <is>
           <t>False</t>
@@ -15396,7 +15416,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0061</t>
+          <t>Sticker-Zen-0062-FIX1</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -15434,14 +15454,10 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>406903249987</t>
-        </is>
-      </c>
-      <c r="K282" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911488570</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr"/>
       <c r="L282" t="inlineStr">
         <is>
           <t>False</t>
@@ -15454,7 +15470,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0061-FIX1</t>
+          <t>Sticker-Zen-0063</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -15492,10 +15508,14 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>406911452547</t>
-        </is>
-      </c>
-      <c r="K283" t="inlineStr"/>
+          <t>406903252007</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="L283" t="inlineStr">
         <is>
           <t>False</t>
@@ -15508,7 +15528,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0062</t>
+          <t>Sticker-Zen-0063-FIX1</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -15546,14 +15566,10 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>406903250891</t>
-        </is>
-      </c>
-      <c r="K284" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911494155</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr"/>
       <c r="L284" t="inlineStr">
         <is>
           <t>False</t>
@@ -15566,7 +15582,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0062-FIX1</t>
+          <t>Sticker-Zen-0066</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -15604,7 +15620,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>406911488570</t>
+          <t>406903252739</t>
         </is>
       </c>
       <c r="K285" t="inlineStr"/>
@@ -15620,7 +15636,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0063</t>
+          <t>Sticker-Zen-0066-FIX1</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -15658,14 +15674,10 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>406903252007</t>
-        </is>
-      </c>
-      <c r="K286" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>406911509730</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr"/>
       <c r="L286" t="inlineStr">
         <is>
           <t>False</t>
@@ -15678,7 +15690,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0063-FIX1</t>
+          <t>Sticker-Zen-0067</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -15714,11 +15726,7 @@
       <c r="I287" t="b">
         <v>1</v>
       </c>
-      <c r="J287" t="inlineStr">
-        <is>
-          <t>406911494155</t>
-        </is>
-      </c>
+      <c r="J287" t="inlineStr"/>
       <c r="K287" t="inlineStr"/>
       <c r="L287" t="inlineStr">
         <is>
@@ -15732,7 +15740,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0066</t>
+          <t>Sticker-Zen-0068</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -15768,11 +15776,7 @@
       <c r="I288" t="b">
         <v>1</v>
       </c>
-      <c r="J288" t="inlineStr">
-        <is>
-          <t>406903252739</t>
-        </is>
-      </c>
+      <c r="J288" t="inlineStr"/>
       <c r="K288" t="inlineStr"/>
       <c r="L288" t="inlineStr">
         <is>
@@ -15786,7 +15790,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0066-FIX1</t>
+          <t>Sticker-Zen-0069</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -15824,7 +15828,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>406911509730</t>
+          <t>406903753067</t>
         </is>
       </c>
       <c r="K289" t="inlineStr"/>
@@ -15840,7 +15844,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0067</t>
+          <t>Sticker-Zen-0069-FIX1</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -15876,7 +15880,11 @@
       <c r="I290" t="b">
         <v>1</v>
       </c>
-      <c r="J290" t="inlineStr"/>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>406911531255</t>
+        </is>
+      </c>
       <c r="K290" t="inlineStr"/>
       <c r="L290" t="inlineStr">
         <is>
@@ -15890,7 +15898,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0068</t>
+          <t>Sticker-Zen-0070</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -15926,7 +15934,11 @@
       <c r="I291" t="b">
         <v>1</v>
       </c>
-      <c r="J291" t="inlineStr"/>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>406903757240</t>
+        </is>
+      </c>
       <c r="K291" t="inlineStr"/>
       <c r="L291" t="inlineStr">
         <is>
@@ -15940,7 +15952,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0069</t>
+          <t>Sticker-Zen-0070-FIX1</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -15978,7 +15990,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>406903753067</t>
+          <t>406911541926</t>
         </is>
       </c>
       <c r="K292" t="inlineStr"/>
@@ -15994,7 +16006,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0069-FIX1</t>
+          <t>Sticker-Zen-0071</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -16032,7 +16044,7 @@
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>406911531255</t>
+          <t>406903762328</t>
         </is>
       </c>
       <c r="K293" t="inlineStr"/>
@@ -16048,7 +16060,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0070</t>
+          <t>Sticker-Zen-0071-FIX1</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -16086,7 +16098,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>406903757240</t>
+          <t>406911551031</t>
         </is>
       </c>
       <c r="K294" t="inlineStr"/>
@@ -16102,7 +16114,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0070-FIX1</t>
+          <t>Sticker-Zen-0072</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -16140,7 +16152,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>406911541926</t>
+          <t>406911942577</t>
         </is>
       </c>
       <c r="K295" t="inlineStr"/>
@@ -16156,7 +16168,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0071</t>
+          <t>Sticker-Zen-0073</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -16194,7 +16206,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>406903762328</t>
+          <t>406911955913</t>
         </is>
       </c>
       <c r="K296" t="inlineStr"/>
@@ -16210,7 +16222,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0071-FIX1</t>
+          <t>Sticker-Zen-0074</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -16248,7 +16260,7 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>406911551031</t>
+          <t>406911953636</t>
         </is>
       </c>
       <c r="K297" t="inlineStr"/>
@@ -16264,7 +16276,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0072</t>
+          <t>Sticker-Zen-0075</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -16302,7 +16314,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>406911942577</t>
+          <t>406912077790</t>
         </is>
       </c>
       <c r="K298" t="inlineStr"/>
@@ -16318,7 +16330,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0073</t>
+          <t>Sticker-Zen-0076</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -16354,11 +16366,7 @@
       <c r="I299" t="b">
         <v>1</v>
       </c>
-      <c r="J299" t="inlineStr">
-        <is>
-          <t>406911955913</t>
-        </is>
-      </c>
+      <c r="J299" t="inlineStr"/>
       <c r="K299" t="inlineStr"/>
       <c r="L299" t="inlineStr">
         <is>
@@ -16372,7 +16380,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Sticker-Zen-0074</t>
+          <t>Sticker-Zen-0081</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -16410,7 +16418,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>406911953636</t>
+          <t>406912094146</t>
         </is>
       </c>
       <c r="K300" t="inlineStr"/>

</xml_diff>